<commit_message>
Chap 7, Ex 28
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,17 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_5391C62B2CDA9FD0DE82F72FEA259FA5AA7038D4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68363713-4C57-4677-9D87-E9A332324241}"/>
   <bookViews>
-    <workbookView windowWidth="19935" windowHeight="7515"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -819,15 +839,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -848,157 +864,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
+      <sz val="9"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1023,194 +898,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1218,335 +907,59 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
+      <font>
+        <b/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1560,24 +973,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1587,43 +983,54 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" name="Order"/>
-    <tableColumn id="2" name="Planned Date"/>
-    <tableColumn id="3" name="Task Type"/>
-    <tableColumn id="4" name="Phase"/>
-    <tableColumn id="5" name="Section(s)"/>
-    <tableColumn id="6" name="Task"/>
-    <tableColumn id="7" name="Exercise"/>
-    <tableColumn id="8" name="Related Result / Reason"/>
-    <tableColumn id="9" name="Prerequisite"/>
-    <tableColumn id="10" name="Proceed Gate"/>
-    <tableColumn id="11" name="Actual Start"/>
-    <tableColumn id="12" name="Actual End"/>
-    <tableColumn id="13" name="First-pass Status"/>
-    <tableColumn id="14" name="Key Blocker"/>
-    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
-    <tableColumn id="16" name="Redo Result"/>
-    <tableColumn id="17" name="Proceed?"/>
-    <tableColumn id="18" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
+      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
+      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" name="First-pass Status"/>
-    <tableColumn id="2" name="Meaning"/>
-    <tableColumn id="3" name="Recommended Action"/>
-    <tableColumn id="4" name="Redo Offset Days"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1772,14 +1179,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1801,7 +1208,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:19">
+    <row r="1" spans="1:19" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1860,7 +1267,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="28.5" spans="1:19">
+    <row r="2" spans="1:19" ht="40.5">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1901,7 +1308,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" ht="28.5" spans="1:19">
+    <row r="3" spans="1:19" ht="40.5">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1942,7 +1349,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:19" ht="27">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -2017,7 +1424,7 @@
         <v>34</v>
       </c>
       <c r="J5" s="6"/>
-      <c r="K5" s="8">
+      <c r="K5" s="7">
         <v>46176</v>
       </c>
       <c r="L5" s="7">
@@ -2039,7 +1446,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:19" ht="27">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2068,7 +1475,7 @@
         <v>38</v>
       </c>
       <c r="J6" s="6"/>
-      <c r="K6" s="8">
+      <c r="K6" s="7">
         <v>46177</v>
       </c>
       <c r="L6" s="7">
@@ -2090,7 +1497,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" ht="28.5" spans="1:19">
+    <row r="7" spans="1:19" ht="27">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2119,7 +1526,7 @@
         <v>44</v>
       </c>
       <c r="J7" s="6"/>
-      <c r="K7" s="8">
+      <c r="K7" s="7">
         <v>46178</v>
       </c>
       <c r="L7" s="7">
@@ -2141,7 +1548,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:19" ht="27">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2273,7 +1680,7 @@
       </c>
       <c r="J10" s="6"/>
       <c r="K10" s="7">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="L10" s="7" t="str">
         <f t="shared" si="0"/>
@@ -2285,7 +1692,7 @@
       <c r="N10" s="6"/>
       <c r="O10" s="7">
         <f>IF(AND($C10="Exercise",$K10&lt;&gt;"",$M10&lt;&gt;""),$K10+VLOOKUP($M10,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="P10" s="7"/>
       <c r="Q10" s="6"/>
@@ -2322,7 +1729,7 @@
       </c>
       <c r="J11" s="6"/>
       <c r="K11" s="7">
-        <v>46188</v>
+        <v>46193</v>
       </c>
       <c r="L11" s="7" t="str">
         <f t="shared" si="0"/>
@@ -2334,14 +1741,14 @@
       <c r="N11" s="6"/>
       <c r="O11" s="7">
         <f>IF(AND($C11="Exercise",$K11&lt;&gt;"",$M11&lt;&gt;""),$K11+VLOOKUP($M11,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v>46190</v>
+        <v>46195</v>
       </c>
       <c r="P11" s="7"/>
       <c r="Q11" s="6"/>
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" ht="28.5" spans="1:19">
+    <row r="12" spans="1:19" ht="40.5">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2370,7 +1777,9 @@
       <c r="J12" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="K12" s="7"/>
+      <c r="K12" s="7">
+        <v>46192</v>
+      </c>
       <c r="L12" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2386,7 +1795,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" ht="28.5" spans="1:19">
+    <row r="13" spans="1:19" ht="27">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2427,7 +1836,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" ht="28.5" spans="1:19">
+    <row r="14" spans="1:19" ht="27">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2472,7 +1881,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" spans="1:19">
+    <row r="15" spans="1:19" ht="27">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2517,7 +1926,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" spans="1:19">
+    <row r="16" spans="1:19" ht="27">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2562,7 +1971,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" spans="1:19">
+    <row r="17" spans="1:19" ht="27">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2607,7 +2016,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" spans="1:19">
+    <row r="18" spans="1:19" ht="27">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2652,7 +2061,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" spans="1:19">
+    <row r="19" spans="1:19" ht="27">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2697,7 +2106,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" spans="1:19">
+    <row r="20" spans="1:19" ht="27">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2742,7 +2151,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" ht="42.75" spans="1:19">
+    <row r="21" spans="1:19" ht="40.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2787,7 +2196,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" ht="28.5" spans="1:19">
+    <row r="22" spans="1:19" ht="40.5">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2828,7 +2237,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" ht="28.5" spans="1:19">
+    <row r="23" spans="1:19" ht="27">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2869,7 +2278,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" spans="1:19">
+    <row r="24" spans="1:19" ht="27">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2914,7 +2323,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" spans="1:19">
+    <row r="25" spans="1:19" ht="27">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -3004,7 +2413,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" ht="28.5" spans="1:19">
+    <row r="27" spans="1:19" ht="27">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -3049,7 +2458,7 @@
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" ht="28.5" spans="1:19">
+    <row r="28" spans="1:19" ht="27">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -3094,7 +2503,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" ht="28.5" spans="1:19">
+    <row r="29" spans="1:19" ht="40.5">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3135,7 +2544,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" ht="28.5" spans="1:19">
+    <row r="30" spans="1:19" ht="27">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3176,7 +2585,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" ht="28.5" spans="1:19">
+    <row r="31" spans="1:19" ht="40.5">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3221,7 +2630,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" ht="28.5" spans="1:19">
+    <row r="32" spans="1:19" ht="40.5">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -3266,7 +2675,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" ht="28.5" spans="1:19">
+    <row r="33" spans="1:19" ht="40.5">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3311,7 +2720,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" ht="28.5" spans="1:19">
+    <row r="34" spans="1:19" ht="40.5">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -3356,7 +2765,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" ht="28.5" spans="1:19">
+    <row r="35" spans="1:19" ht="40.5">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3401,7 +2810,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" ht="28.5" spans="1:19">
+    <row r="36" spans="1:19" ht="40.5">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -3446,7 +2855,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" ht="28.5" spans="1:19">
+    <row r="37" spans="1:19" ht="40.5">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3491,7 +2900,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" ht="28.5" spans="1:19">
+    <row r="38" spans="1:19" ht="40.5">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3536,7 +2945,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" ht="28.5" spans="1:19">
+    <row r="39" spans="1:19" ht="40.5">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3581,7 +2990,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" ht="28.5" spans="1:19">
+    <row r="40" spans="1:19" ht="40.5">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3626,7 +3035,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" ht="28.5" spans="1:19">
+    <row r="41" spans="1:19" ht="40.5">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3671,7 +3080,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" ht="28.5" spans="1:19">
+    <row r="42" spans="1:19" ht="40.5">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3712,7 +3121,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" ht="28.5" spans="1:19">
+    <row r="43" spans="1:19" ht="40.5">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3753,7 +3162,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" ht="28.5" spans="1:19">
+    <row r="44" spans="1:19" ht="40.5">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3798,7 +3207,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" ht="28.5" spans="1:19">
+    <row r="45" spans="1:19" ht="40.5">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3843,7 +3252,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" ht="28.5" spans="1:19">
+    <row r="46" spans="1:19" ht="40.5">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3888,7 +3297,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" ht="28.5" spans="1:19">
+    <row r="47" spans="1:19" ht="40.5">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3933,7 +3342,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" ht="28.5" spans="1:19">
+    <row r="48" spans="1:19" ht="40.5">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3978,7 +3387,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" ht="28.5" spans="1:19">
+    <row r="49" spans="1:19" ht="40.5">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -4023,7 +3432,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" ht="28.5" spans="1:19">
+    <row r="50" spans="1:19" ht="40.5">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -4068,7 +3477,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" ht="28.5" spans="1:19">
+    <row r="51" spans="1:19" ht="40.5">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -4113,7 +3522,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" ht="28.5" spans="1:19">
+    <row r="52" spans="1:19" ht="40.5">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -4158,7 +3567,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" ht="28.5" spans="1:19">
+    <row r="53" spans="1:19" ht="40.5">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -4203,7 +3612,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" ht="28.5" spans="1:19">
+    <row r="54" spans="1:19" ht="40.5">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -4248,7 +3657,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" ht="28.5" spans="1:19">
+    <row r="55" spans="1:19" ht="40.5">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -4293,7 +3702,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" ht="28.5" spans="1:19">
+    <row r="56" spans="1:19" ht="40.5">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -4338,7 +3747,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" ht="42.75" spans="1:19">
+    <row r="57" spans="1:19" ht="40.5">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -4379,7 +3788,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" ht="28.5" spans="1:19">
+    <row r="58" spans="1:19" ht="27">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4424,7 +3833,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" ht="28.5" spans="1:19">
+    <row r="59" spans="1:19" ht="27">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4469,7 +3878,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" ht="28.5" spans="1:19">
+    <row r="60" spans="1:19" ht="27">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4514,7 +3923,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" ht="28.5" spans="1:19">
+    <row r="61" spans="1:19" ht="27">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4559,7 +3968,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" ht="28.5" spans="1:19">
+    <row r="62" spans="1:19" ht="27">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4604,7 +4013,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" ht="42.75" spans="1:19">
+    <row r="63" spans="1:19" ht="40.5">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4645,7 +4054,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" ht="42.75" spans="1:19">
+    <row r="64" spans="1:19" ht="40.5">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4687,35 +4096,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64">
+    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64">
+    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4723,22 +4132,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" spans="1:2">
+    <row r="1" spans="1:2" ht="27">
       <c r="A1" s="1" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" ht="28.5" spans="1:2">
+    <row r="2" spans="1:2" ht="27">
       <c r="A2" s="3" t="s">
         <v>238</v>
       </c>
@@ -4750,7 +4158,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" ht="15" spans="1:2">
+    <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>240</v>
       </c>
@@ -4759,7 +4167,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="15" spans="1:2">
+    <row r="5" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>241</v>
       </c>
@@ -4768,7 +4176,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="15" spans="1:2">
+    <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>242</v>
       </c>
@@ -4777,7 +4185,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" ht="15" spans="1:2">
+    <row r="7" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>243</v>
       </c>
@@ -4786,7 +4194,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="15" spans="1:2">
+    <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>244</v>
       </c>
@@ -4795,7 +4203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15" spans="1:2">
+    <row r="9" spans="1:2" ht="27">
       <c r="A9" s="5" t="s">
         <v>245</v>
       </c>
@@ -4804,20 +4212,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" ht="15" spans="1:2">
+    <row r="10" spans="1:2" ht="27">
       <c r="A10" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" ht="15" spans="1:2">
+    <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>247</v>
       </c>
@@ -4826,7 +4234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="15" spans="1:2">
+    <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -4835,7 +4243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" ht="15" spans="1:2">
+    <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -4844,7 +4252,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" ht="15" spans="1:2">
+    <row r="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
@@ -4857,7 +4265,7 @@
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" ht="15" spans="1:2">
+    <row r="17" spans="1:2" ht="27">
       <c r="A17" s="5" t="s">
         <v>248</v>
       </c>
@@ -4865,7 +4273,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="18" ht="15" spans="1:2">
+    <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>250</v>
       </c>
@@ -4874,16 +4282,15 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4891,7 +4298,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:4">
+    <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -4961,7 +4368,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>263</v>
       </c>
@@ -4973,8 +4380,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7 process update
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_5391C62B2CDA9FD0DE82F72FEA259FA5AA7038D4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68363713-4C57-4677-9D87-E9A332324241}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="14_{58114150-BD7F-4246-9469-DE5FA7D62A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{314821D1-A16E-49A6-9BF3-7E6E9A5F809A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1620" yWindow="3015" windowWidth="25245" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -1192,12 +1192,12 @@
     <col min="2" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="50" customWidth="1"/>
+    <col min="6" max="6" width="37.5" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="8" max="8" width="19.875" customWidth="1"/>
     <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="28" customWidth="1"/>
-    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="10" max="10" width="18.375" customWidth="1"/>
+    <col min="11" max="11" width="17.875" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
     <col min="14" max="14" width="28" customWidth="1"/>
@@ -1267,7 +1267,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="40.5">
+    <row r="2" spans="1:19" ht="54">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1308,7 +1308,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" spans="1:19" ht="40.5">
+    <row r="3" spans="1:19" ht="54">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:19" ht="27">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1599,7 +1599,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:19" ht="27">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1650,7 +1650,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" ht="27">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -1682,9 +1682,9 @@
       <c r="K10" s="7">
         <v>46188</v>
       </c>
-      <c r="L10" s="7" t="str">
+      <c r="L10" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46194</v>
       </c>
       <c r="M10" s="6" t="s">
         <v>55</v>
@@ -1694,12 +1694,14 @@
         <f>IF(AND($C10="Exercise",$K10&lt;&gt;"",$M10&lt;&gt;""),$K10+VLOOKUP($M10,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46190</v>
       </c>
-      <c r="P10" s="7"/>
+      <c r="P10" s="7">
+        <v>46194</v>
+      </c>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:19" ht="27">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1731,9 +1733,9 @@
       <c r="K11" s="7">
         <v>46193</v>
       </c>
-      <c r="L11" s="7" t="str">
+      <c r="L11" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46194</v>
       </c>
       <c r="M11" s="6" t="s">
         <v>39</v>
@@ -1743,12 +1745,14 @@
         <f>IF(AND($C11="Exercise",$K11&lt;&gt;"",$M11&lt;&gt;""),$K11+VLOOKUP($M11,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46195</v>
       </c>
-      <c r="P11" s="7"/>
+      <c r="P11" s="7">
+        <v>46194</v>
+      </c>
       <c r="Q11" s="6"/>
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" spans="1:19" ht="40.5">
+    <row r="12" spans="1:19" ht="54">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -1780,9 +1784,9 @@
       <c r="K12" s="7">
         <v>46192</v>
       </c>
-      <c r="L12" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="L12" s="7">
+        <f>IF($P12&lt;&gt;"",$P12,"")</f>
+        <v>46192</v>
       </c>
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
@@ -1790,12 +1794,14 @@
         <f>IF(AND($C12="Exercise",$K12&lt;&gt;"",$M12&lt;&gt;""),$K12+VLOOKUP($M12,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v/>
       </c>
-      <c r="P12" s="7"/>
+      <c r="P12" s="7">
+        <v>46192</v>
+      </c>
       <c r="Q12" s="6"/>
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" spans="1:19" ht="27">
+    <row r="13" spans="1:19" ht="40.5">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1820,10 +1826,11 @@
         <v>68</v>
       </c>
       <c r="J13" s="6"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="K13" s="7">
+        <v>46194</v>
+      </c>
+      <c r="L13" s="7">
+        <v>46195</v>
       </c>
       <c r="M13" s="6"/>
       <c r="N13" s="6"/>
@@ -1836,7 +1843,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" spans="1:19" ht="27">
+    <row r="14" spans="1:19" ht="40.5">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -1971,7 +1978,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" spans="1:19" ht="27">
+    <row r="17" spans="1:19" ht="40.5">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2016,7 +2023,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" spans="1:19" ht="27">
+    <row r="18" spans="1:19" ht="40.5">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2151,7 +2158,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" spans="1:19" ht="40.5">
+    <row r="21" spans="1:19" ht="67.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2237,7 +2244,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" spans="1:19" ht="27">
+    <row r="23" spans="1:19" ht="40.5">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2278,7 +2285,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" spans="1:19" ht="27">
+    <row r="24" spans="1:19" ht="40.5">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2368,7 +2375,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" spans="1:19">
+    <row r="26" spans="1:19" ht="27">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -2413,7 +2420,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" spans="1:19" ht="27">
+    <row r="27" spans="1:19" ht="40.5">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2458,7 +2465,7 @@
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" spans="1:19" ht="27">
+    <row r="28" spans="1:19" ht="40.5">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -2503,7 +2510,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" spans="1:19" ht="40.5">
+    <row r="29" spans="1:19" ht="54">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -2544,7 +2551,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" spans="1:19" ht="27">
+    <row r="30" spans="1:19" ht="40.5">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3035,7 +3042,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" spans="1:19" ht="40.5">
+    <row r="41" spans="1:19" ht="54">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3080,7 +3087,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" spans="1:19" ht="40.5">
+    <row r="42" spans="1:19" ht="54">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3702,7 +3709,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" spans="1:19" ht="40.5">
+    <row r="56" spans="1:19" ht="54">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -3747,7 +3754,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" spans="1:19" ht="40.5">
+    <row r="57" spans="1:19" ht="67.5">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -3788,7 +3795,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" spans="1:19" ht="27">
+    <row r="58" spans="1:19" ht="40.5">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4013,7 +4020,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" spans="1:19" ht="40.5">
+    <row r="63" spans="1:19" ht="54">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4054,7 +4061,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" spans="1:19" ht="40.5">
+    <row r="64" spans="1:19" ht="54">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4209,7 +4216,7 @@
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="27">
@@ -4218,7 +4225,7 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:2">

</xml_diff>

<commit_message>
Chap 7, Ex 5
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,42 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="14_{58114150-BD7F-4246-9469-DE5FA7D62A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{314821D1-A16E-49A6-9BF3-7E6E9A5F809A}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="3015" windowWidth="25245" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="28245" windowHeight="12465"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="266">
   <si>
     <t>Order</t>
   </si>
@@ -839,11 +819,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -864,16 +848,157 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Carlito"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Carlito"/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -898,8 +1023,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -907,52 +1218,339 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+  <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <font>
-        <b/>
-      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -966,14 +1564,17 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFE699"/>
+          <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="1"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -983,54 +1584,43 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
-      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
-      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
+    <tableColumn id="1" name="Order"/>
+    <tableColumn id="2" name="Planned Date"/>
+    <tableColumn id="3" name="Task Type"/>
+    <tableColumn id="4" name="Phase"/>
+    <tableColumn id="5" name="Section(s)"/>
+    <tableColumn id="6" name="Task"/>
+    <tableColumn id="7" name="Exercise"/>
+    <tableColumn id="8" name="Related Result / Reason"/>
+    <tableColumn id="9" name="Prerequisite"/>
+    <tableColumn id="10" name="Proceed Gate"/>
+    <tableColumn id="11" name="Actual Start"/>
+    <tableColumn id="12" name="Actual End"/>
+    <tableColumn id="13" name="First-pass Status"/>
+    <tableColumn id="14" name="Key Blocker"/>
+    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
+    <tableColumn id="16" name="Redo Result"/>
+    <tableColumn id="17" name="Proceed?"/>
+    <tableColumn id="18" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
+    <tableColumn id="1" name="First-pass Status"/>
+    <tableColumn id="2" name="Meaning"/>
+    <tableColumn id="3" name="Recommended Action"/>
+    <tableColumn id="4" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1179,14 +1769,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1208,7 +1798,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="32.1" customHeight="1">
+    <row r="1" ht="32.1" customHeight="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1267,7 +1857,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="54">
+    <row r="2" ht="42.75" spans="1:19">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1308,7 +1898,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" spans="1:19" ht="54">
+    <row r="3" ht="42.75" spans="1:19">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1349,7 +1939,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" spans="1:19" ht="27">
+    <row r="4" ht="28.5" spans="1:19">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1395,7 +1985,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" spans="1:19" ht="27">
+    <row r="5" ht="28.5" spans="1:19">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1446,7 +2036,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" spans="1:19" ht="27">
+    <row r="6" ht="28.5" spans="1:19">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -1497,7 +2087,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" spans="1:19" ht="27">
+    <row r="7" ht="28.5" spans="1:19">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -1548,7 +2138,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" spans="1:19" ht="27">
+    <row r="8" ht="28.5" spans="1:19">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -1599,7 +2189,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" spans="1:19" ht="27">
+    <row r="9" ht="28.5" spans="1:19">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1650,7 +2240,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19" ht="27">
+    <row r="10" spans="1:19">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -1701,7 +2291,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" spans="1:19" ht="27">
+    <row r="11" ht="28.5" spans="1:19">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1752,7 +2342,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" spans="1:19" ht="54">
+    <row r="12" ht="57" spans="1:19">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -1785,7 +2375,7 @@
         <v>46192</v>
       </c>
       <c r="L12" s="7">
-        <f>IF($P12&lt;&gt;"",$P12,"")</f>
+        <f t="shared" si="0"/>
         <v>46192</v>
       </c>
       <c r="M12" s="6"/>
@@ -1801,7 +2391,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" spans="1:19" ht="40.5">
+    <row r="13" ht="42.75" spans="1:19">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1843,7 +2433,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" spans="1:19" ht="40.5">
+    <row r="14" ht="28.5" spans="1:19">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -1872,23 +2462,29 @@
         <v>71</v>
       </c>
       <c r="J14" s="6"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7" t="str">
+      <c r="K14" s="7">
+        <v>46196</v>
+      </c>
+      <c r="L14" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="M14" s="6"/>
+        <v>46199</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N14" s="6"/>
-      <c r="O14" s="7" t="str">
+      <c r="O14" s="7">
         <f>IF(AND($C14="Exercise",$K14&lt;&gt;"",$M14&lt;&gt;""),$K14+VLOOKUP($M14,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="P14" s="7"/>
+        <v>46198</v>
+      </c>
+      <c r="P14" s="7">
+        <v>46199</v>
+      </c>
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" spans="1:19" ht="27">
+    <row r="15" ht="28.5" spans="1:19">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1917,23 +2513,27 @@
         <v>75</v>
       </c>
       <c r="J15" s="6"/>
-      <c r="K15" s="7"/>
+      <c r="K15" s="7">
+        <v>46197</v>
+      </c>
       <c r="L15" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M15" s="6"/>
+      <c r="M15" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N15" s="6"/>
-      <c r="O15" s="7" t="str">
+      <c r="O15" s="7">
         <f>IF(AND($C15="Exercise",$K15&lt;&gt;"",$M15&lt;&gt;""),$K15+VLOOKUP($M15,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46199</v>
       </c>
       <c r="P15" s="7"/>
       <c r="Q15" s="6"/>
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" spans="1:19" ht="27">
+    <row r="16" ht="28.5" spans="1:19">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -1978,7 +2578,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" spans="1:19" ht="40.5">
+    <row r="17" ht="28.5" spans="1:19">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2023,7 +2623,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" spans="1:19" ht="40.5">
+    <row r="18" ht="28.5" spans="1:19">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2068,7 +2668,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" spans="1:19" ht="27">
+    <row r="19" ht="28.5" spans="1:19">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2113,7 +2713,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" spans="1:19" ht="27">
+    <row r="20" ht="28.5" spans="1:19">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2158,7 +2758,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" spans="1:19" ht="67.5">
+    <row r="21" ht="57" spans="1:19">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2203,7 +2803,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" spans="1:19" ht="40.5">
+    <row r="22" ht="42.75" spans="1:19">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2244,7 +2844,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" spans="1:19" ht="40.5">
+    <row r="23" ht="42.75" spans="1:19">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2285,7 +2885,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" spans="1:19" ht="40.5">
+    <row r="24" ht="28.5" spans="1:19">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2330,7 +2930,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" spans="1:19" ht="27">
+    <row r="25" ht="28.5" spans="1:19">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2375,7 +2975,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" spans="1:19" ht="27">
+    <row r="26" ht="28.5" spans="1:19">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -2420,7 +3020,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" spans="1:19" ht="40.5">
+    <row r="27" ht="28.5" spans="1:19">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2465,7 +3065,7 @@
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" spans="1:19" ht="40.5">
+    <row r="28" ht="42.75" spans="1:19">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -2510,7 +3110,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" spans="1:19" ht="54">
+    <row r="29" ht="42.75" spans="1:19">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -2551,7 +3151,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" spans="1:19" ht="40.5">
+    <row r="30" ht="28.5" spans="1:19">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -2592,7 +3192,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" spans="1:19" ht="40.5">
+    <row r="31" ht="28.5" spans="1:19">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -2637,7 +3237,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" spans="1:19" ht="40.5">
+    <row r="32" ht="28.5" spans="1:19">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -2682,7 +3282,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" spans="1:19" ht="40.5">
+    <row r="33" ht="28.5" spans="1:19">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -2727,7 +3327,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" spans="1:19" ht="40.5">
+    <row r="34" ht="28.5" spans="1:19">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -2772,7 +3372,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" spans="1:19" ht="40.5">
+    <row r="35" ht="28.5" spans="1:19">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2817,7 +3417,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" spans="1:19" ht="40.5">
+    <row r="36" ht="28.5" spans="1:19">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -2862,7 +3462,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" spans="1:19" ht="40.5">
+    <row r="37" ht="28.5" spans="1:19">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2907,7 +3507,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" spans="1:19" ht="40.5">
+    <row r="38" ht="28.5" spans="1:19">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -2952,7 +3552,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" spans="1:19" ht="40.5">
+    <row r="39" ht="28.5" spans="1:19">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -2997,7 +3597,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" spans="1:19" ht="40.5">
+    <row r="40" ht="28.5" spans="1:19">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3042,7 +3642,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" spans="1:19" ht="54">
+    <row r="41" ht="42.75" spans="1:19">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3087,7 +3687,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" spans="1:19" ht="54">
+    <row r="42" ht="42.75" spans="1:19">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3128,7 +3728,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" spans="1:19" ht="40.5">
+    <row r="43" ht="42.75" spans="1:19">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3169,7 +3769,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" spans="1:19" ht="40.5">
+    <row r="44" ht="28.5" spans="1:19">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3214,7 +3814,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" spans="1:19" ht="40.5">
+    <row r="45" ht="28.5" spans="1:19">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3259,7 +3859,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" spans="1:19" ht="40.5">
+    <row r="46" ht="28.5" spans="1:19">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3304,7 +3904,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" spans="1:19" ht="40.5">
+    <row r="47" ht="28.5" spans="1:19">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3349,7 +3949,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" spans="1:19" ht="40.5">
+    <row r="48" ht="28.5" spans="1:19">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3394,7 +3994,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" spans="1:19" ht="40.5">
+    <row r="49" ht="28.5" spans="1:19">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -3439,7 +4039,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" spans="1:19" ht="40.5">
+    <row r="50" ht="28.5" spans="1:19">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -3484,7 +4084,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" spans="1:19" ht="40.5">
+    <row r="51" ht="28.5" spans="1:19">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -3529,7 +4129,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" spans="1:19" ht="40.5">
+    <row r="52" ht="28.5" spans="1:19">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -3574,7 +4174,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" spans="1:19" ht="40.5">
+    <row r="53" ht="28.5" spans="1:19">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -3619,7 +4219,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" spans="1:19" ht="40.5">
+    <row r="54" ht="28.5" spans="1:19">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -3664,7 +4264,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" spans="1:19" ht="40.5">
+    <row r="55" ht="28.5" spans="1:19">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -3709,7 +4309,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" spans="1:19" ht="54">
+    <row r="56" ht="42.75" spans="1:19">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -3754,7 +4354,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" spans="1:19" ht="67.5">
+    <row r="57" ht="57" spans="1:19">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -3795,7 +4395,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" spans="1:19" ht="40.5">
+    <row r="58" ht="28.5" spans="1:19">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -3840,7 +4440,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" spans="1:19" ht="27">
+    <row r="59" ht="28.5" spans="1:19">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -3885,7 +4485,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" spans="1:19" ht="27">
+    <row r="60" ht="28.5" spans="1:19">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -3930,7 +4530,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" spans="1:19" ht="27">
+    <row r="61" ht="28.5" spans="1:19">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -3975,7 +4575,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" spans="1:19" ht="27">
+    <row r="62" ht="28.5" spans="1:19">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4020,7 +4620,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" spans="1:19" ht="54">
+    <row r="63" ht="42.75" spans="1:19">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4061,7 +4661,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" spans="1:19" ht="54">
+    <row r="64" ht="57" spans="1:19">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4103,35 +4703,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="M2:M64">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="Q2:R64">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4139,21 +4739,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="27">
+    <row r="1" ht="30" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="27">
+    <row r="2" ht="28.5" spans="1:2">
       <c r="A2" s="3" t="s">
         <v>238</v>
       </c>
@@ -4165,7 +4766,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" ht="15" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>240</v>
       </c>
@@ -4174,7 +4775,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" ht="15" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>241</v>
       </c>
@@ -4183,7 +4784,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" ht="15" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>242</v>
       </c>
@@ -4192,7 +4793,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" ht="15" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>243</v>
       </c>
@@ -4201,7 +4802,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" ht="15" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>244</v>
       </c>
@@ -4210,29 +4811,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="27">
+    <row r="9" ht="15" spans="1:2">
       <c r="A9" s="5" t="s">
         <v>245</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="27">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" ht="15" spans="1:2">
       <c r="A10" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" ht="15" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>247</v>
       </c>
@@ -4241,7 +4842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" ht="15" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -4250,16 +4851,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" ht="15" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" ht="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
@@ -4272,7 +4873,7 @@
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" spans="1:2" ht="27">
+    <row r="17" ht="15" spans="1:2">
       <c r="A17" s="5" t="s">
         <v>248</v>
       </c>
@@ -4280,7 +4881,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" ht="15" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>250</v>
       </c>
@@ -4289,15 +4890,16 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4305,7 +4907,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27">
+    <row r="1" ht="15" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -4375,7 +4977,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>263</v>
       </c>
@@ -4387,8 +4989,8 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, Ex 7
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,22 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="14_{07D48870-0C2D-4C3F-95EC-9B844142D55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECA2C51C-270F-494F-85CE-669E444192F2}"/>
   <bookViews>
-    <workbookView windowWidth="28245" windowHeight="12465"/>
+    <workbookView xWindow="2655" yWindow="4050" windowWidth="25245" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="266">
   <si>
     <t>Order</t>
   </si>
@@ -819,15 +839,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -848,157 +864,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
+      <sz val="9"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1023,194 +898,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1218,332 +907,59 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
+      <font>
+        <b/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1557,24 +973,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1584,43 +983,54 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" name="Order"/>
-    <tableColumn id="2" name="Planned Date"/>
-    <tableColumn id="3" name="Task Type"/>
-    <tableColumn id="4" name="Phase"/>
-    <tableColumn id="5" name="Section(s)"/>
-    <tableColumn id="6" name="Task"/>
-    <tableColumn id="7" name="Exercise"/>
-    <tableColumn id="8" name="Related Result / Reason"/>
-    <tableColumn id="9" name="Prerequisite"/>
-    <tableColumn id="10" name="Proceed Gate"/>
-    <tableColumn id="11" name="Actual Start"/>
-    <tableColumn id="12" name="Actual End"/>
-    <tableColumn id="13" name="First-pass Status"/>
-    <tableColumn id="14" name="Key Blocker"/>
-    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
-    <tableColumn id="16" name="Redo Result"/>
-    <tableColumn id="17" name="Proceed?"/>
-    <tableColumn id="18" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
+      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
+      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" name="First-pass Status"/>
-    <tableColumn id="2" name="Meaning"/>
-    <tableColumn id="3" name="Recommended Action"/>
-    <tableColumn id="4" name="Redo Offset Days"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1769,14 +1179,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1798,7 +1208,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:19">
+    <row r="1" spans="1:19" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1857,7 +1267,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="42.75" spans="1:19">
+    <row r="2" spans="1:19" ht="54">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1898,7 +1308,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" ht="42.75" spans="1:19">
+    <row r="3" spans="1:19" ht="54">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1939,7 +1349,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" ht="28.5" spans="1:19">
+    <row r="4" spans="1:19" ht="27">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1985,7 +1395,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" ht="28.5" spans="1:19">
+    <row r="5" spans="1:19" ht="27">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2036,7 +1446,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" ht="28.5" spans="1:19">
+    <row r="6" spans="1:19" ht="27">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2087,7 +1497,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" ht="28.5" spans="1:19">
+    <row r="7" spans="1:19" ht="27">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2138,7 +1548,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" ht="28.5" spans="1:19">
+    <row r="8" spans="1:19" ht="27">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2189,7 +1599,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" ht="28.5" spans="1:19">
+    <row r="9" spans="1:19" ht="27">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2240,7 +1650,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" ht="27">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2291,7 +1701,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" ht="28.5" spans="1:19">
+    <row r="11" spans="1:19" ht="27">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2342,7 +1752,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" ht="57" spans="1:19">
+    <row r="12" spans="1:19" ht="54">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2391,7 +1801,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" ht="42.75" spans="1:19">
+    <row r="13" spans="1:19" ht="40.5">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2433,7 +1843,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" ht="28.5" spans="1:19">
+    <row r="14" spans="1:19" ht="40.5">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2484,7 +1894,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" ht="28.5" spans="1:19">
+    <row r="15" spans="1:19" ht="27">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2533,7 +1943,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" ht="28.5" spans="1:19">
+    <row r="16" spans="1:19" ht="27">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2562,23 +1972,27 @@
         <v>79</v>
       </c>
       <c r="J16" s="6"/>
-      <c r="K16" s="7"/>
+      <c r="K16" s="7">
+        <v>46201</v>
+      </c>
       <c r="L16" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M16" s="6"/>
+      <c r="M16" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="N16" s="6"/>
-      <c r="O16" s="7" t="str">
+      <c r="O16" s="7">
         <f>IF(AND($C16="Exercise",$K16&lt;&gt;"",$M16&lt;&gt;""),$K16+VLOOKUP($M16,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46203</v>
       </c>
       <c r="P16" s="7"/>
       <c r="Q16" s="6"/>
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" ht="28.5" spans="1:19">
+    <row r="17" spans="1:19" ht="40.5">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2623,7 +2037,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" ht="28.5" spans="1:19">
+    <row r="18" spans="1:19" ht="40.5">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2668,7 +2082,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" ht="28.5" spans="1:19">
+    <row r="19" spans="1:19" ht="27">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2713,7 +2127,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" ht="28.5" spans="1:19">
+    <row r="20" spans="1:19" ht="27">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2758,7 +2172,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" ht="57" spans="1:19">
+    <row r="21" spans="1:19" ht="67.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2803,7 +2217,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" ht="42.75" spans="1:19">
+    <row r="22" spans="1:19" ht="40.5">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2844,7 +2258,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" ht="42.75" spans="1:19">
+    <row r="23" spans="1:19" ht="40.5">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2885,7 +2299,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" ht="28.5" spans="1:19">
+    <row r="24" spans="1:19" ht="40.5">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2930,7 +2344,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" ht="28.5" spans="1:19">
+    <row r="25" spans="1:19" ht="27">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2975,7 +2389,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" ht="28.5" spans="1:19">
+    <row r="26" spans="1:19" ht="27">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -3020,7 +2434,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" ht="28.5" spans="1:19">
+    <row r="27" spans="1:19" ht="40.5">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -3065,7 +2479,7 @@
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" ht="42.75" spans="1:19">
+    <row r="28" spans="1:19" ht="40.5">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -3110,7 +2524,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" ht="42.75" spans="1:19">
+    <row r="29" spans="1:19" ht="54">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3151,7 +2565,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" ht="28.5" spans="1:19">
+    <row r="30" spans="1:19" ht="40.5">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3192,7 +2606,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" ht="28.5" spans="1:19">
+    <row r="31" spans="1:19" ht="40.5">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3237,7 +2651,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" ht="28.5" spans="1:19">
+    <row r="32" spans="1:19" ht="40.5">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -3282,7 +2696,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" ht="28.5" spans="1:19">
+    <row r="33" spans="1:19" ht="40.5">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3327,7 +2741,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" ht="28.5" spans="1:19">
+    <row r="34" spans="1:19" ht="40.5">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -3372,7 +2786,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" ht="28.5" spans="1:19">
+    <row r="35" spans="1:19" ht="40.5">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3417,7 +2831,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" ht="28.5" spans="1:19">
+    <row r="36" spans="1:19" ht="40.5">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -3462,7 +2876,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" ht="28.5" spans="1:19">
+    <row r="37" spans="1:19" ht="40.5">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3507,7 +2921,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" ht="28.5" spans="1:19">
+    <row r="38" spans="1:19" ht="40.5">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3552,7 +2966,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" ht="28.5" spans="1:19">
+    <row r="39" spans="1:19" ht="40.5">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3597,7 +3011,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" ht="28.5" spans="1:19">
+    <row r="40" spans="1:19" ht="40.5">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3642,7 +3056,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" ht="42.75" spans="1:19">
+    <row r="41" spans="1:19" ht="54">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3687,7 +3101,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" ht="42.75" spans="1:19">
+    <row r="42" spans="1:19" ht="54">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3728,7 +3142,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" ht="42.75" spans="1:19">
+    <row r="43" spans="1:19" ht="40.5">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3769,7 +3183,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" ht="28.5" spans="1:19">
+    <row r="44" spans="1:19" ht="40.5">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3814,7 +3228,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" ht="28.5" spans="1:19">
+    <row r="45" spans="1:19" ht="40.5">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3859,7 +3273,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" ht="28.5" spans="1:19">
+    <row r="46" spans="1:19" ht="40.5">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3904,7 +3318,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" ht="28.5" spans="1:19">
+    <row r="47" spans="1:19" ht="40.5">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3949,7 +3363,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" ht="28.5" spans="1:19">
+    <row r="48" spans="1:19" ht="40.5">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3994,7 +3408,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" ht="28.5" spans="1:19">
+    <row r="49" spans="1:19" ht="40.5">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -4039,7 +3453,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" ht="28.5" spans="1:19">
+    <row r="50" spans="1:19" ht="40.5">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -4084,7 +3498,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" ht="28.5" spans="1:19">
+    <row r="51" spans="1:19" ht="40.5">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -4129,7 +3543,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" ht="28.5" spans="1:19">
+    <row r="52" spans="1:19" ht="40.5">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -4174,7 +3588,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" ht="28.5" spans="1:19">
+    <row r="53" spans="1:19" ht="40.5">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -4219,7 +3633,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" ht="28.5" spans="1:19">
+    <row r="54" spans="1:19" ht="40.5">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -4264,7 +3678,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" ht="28.5" spans="1:19">
+    <row r="55" spans="1:19" ht="40.5">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -4309,7 +3723,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" ht="42.75" spans="1:19">
+    <row r="56" spans="1:19" ht="54">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -4354,7 +3768,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" ht="57" spans="1:19">
+    <row r="57" spans="1:19" ht="67.5">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -4395,7 +3809,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" ht="28.5" spans="1:19">
+    <row r="58" spans="1:19" ht="40.5">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4440,7 +3854,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" ht="28.5" spans="1:19">
+    <row r="59" spans="1:19" ht="27">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4485,7 +3899,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" ht="28.5" spans="1:19">
+    <row r="60" spans="1:19" ht="27">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4530,7 +3944,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" ht="28.5" spans="1:19">
+    <row r="61" spans="1:19" ht="27">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4575,7 +3989,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" ht="28.5" spans="1:19">
+    <row r="62" spans="1:19" ht="27">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4620,7 +4034,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" ht="42.75" spans="1:19">
+    <row r="63" spans="1:19" ht="54">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4661,7 +4075,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" ht="57" spans="1:19">
+    <row r="64" spans="1:19" ht="54">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4703,35 +4117,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64">
+    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64">
+    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4739,22 +4153,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" spans="1:2">
+    <row r="1" spans="1:2" ht="27">
       <c r="A1" s="1" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" ht="28.5" spans="1:2">
+    <row r="2" spans="1:2" ht="27">
       <c r="A2" s="3" t="s">
         <v>238</v>
       </c>
@@ -4766,7 +4179,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" ht="15" spans="1:2">
+    <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>240</v>
       </c>
@@ -4775,7 +4188,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="15" spans="1:2">
+    <row r="5" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>241</v>
       </c>
@@ -4784,7 +4197,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="15" spans="1:2">
+    <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>242</v>
       </c>
@@ -4793,7 +4206,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" ht="15" spans="1:2">
+    <row r="7" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>243</v>
       </c>
@@ -4802,7 +4215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="15" spans="1:2">
+    <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>244</v>
       </c>
@@ -4811,7 +4224,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15" spans="1:2">
+    <row r="9" spans="1:2" ht="27">
       <c r="A9" s="5" t="s">
         <v>245</v>
       </c>
@@ -4820,20 +4233,20 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" ht="15" spans="1:2">
+    <row r="10" spans="1:2" ht="27">
       <c r="A10" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" ht="15" spans="1:2">
+    <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>247</v>
       </c>
@@ -4842,16 +4255,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="15" spans="1:2">
+    <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Spark")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="15" spans="1:2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -4860,7 +4273,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" ht="15" spans="1:2">
+    <row r="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
@@ -4873,7 +4286,7 @@
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" ht="15" spans="1:2">
+    <row r="17" spans="1:2" ht="27">
       <c r="A17" s="5" t="s">
         <v>248</v>
       </c>
@@ -4881,7 +4294,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="18" ht="15" spans="1:2">
+    <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>250</v>
       </c>
@@ -4890,16 +4303,15 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4907,7 +4319,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:4">
+    <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -4977,7 +4389,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>263</v>
       </c>
@@ -4989,8 +4401,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, Ex 34
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,42 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="14_{07D48870-0C2D-4C3F-95EC-9B844142D55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECA2C51C-270F-494F-85CE-669E444192F2}"/>
   <bookViews>
-    <workbookView xWindow="2655" yWindow="4050" windowWidth="25245" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="28245" windowHeight="12465"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="266">
   <si>
     <t>Order</t>
   </si>
@@ -839,11 +819,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -864,16 +848,157 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Carlito"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Carlito"/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -898,8 +1023,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -907,52 +1218,339 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+  <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <font>
-        <b/>
-      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -966,14 +1564,17 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFE699"/>
+          <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="1"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -983,54 +1584,43 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
-      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
-      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
+    <tableColumn id="1" name="Order"/>
+    <tableColumn id="2" name="Planned Date"/>
+    <tableColumn id="3" name="Task Type"/>
+    <tableColumn id="4" name="Phase"/>
+    <tableColumn id="5" name="Section(s)"/>
+    <tableColumn id="6" name="Task"/>
+    <tableColumn id="7" name="Exercise"/>
+    <tableColumn id="8" name="Related Result / Reason"/>
+    <tableColumn id="9" name="Prerequisite"/>
+    <tableColumn id="10" name="Proceed Gate"/>
+    <tableColumn id="11" name="Actual Start"/>
+    <tableColumn id="12" name="Actual End"/>
+    <tableColumn id="13" name="First-pass Status"/>
+    <tableColumn id="14" name="Key Blocker"/>
+    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
+    <tableColumn id="16" name="Redo Result"/>
+    <tableColumn id="17" name="Proceed?"/>
+    <tableColumn id="18" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
+    <tableColumn id="1" name="First-pass Status"/>
+    <tableColumn id="2" name="Meaning"/>
+    <tableColumn id="3" name="Recommended Action"/>
+    <tableColumn id="4" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1179,14 +1769,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1195,7 +1785,7 @@
     <col min="6" max="6" width="37.5" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="19.875" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="9" max="9" width="21.75" customWidth="1"/>
     <col min="10" max="10" width="18.375" customWidth="1"/>
     <col min="11" max="11" width="17.875" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
@@ -1208,7 +1798,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="32.1" customHeight="1">
+    <row r="1" ht="32.1" customHeight="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1267,7 +1857,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="54">
+    <row r="2" ht="42.75" spans="1:19">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1308,7 +1898,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" spans="1:19" ht="54">
+    <row r="3" ht="42.75" spans="1:19">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1349,7 +1939,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" spans="1:19" ht="27">
+    <row r="4" ht="28.5" spans="1:19">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1395,7 +1985,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" spans="1:19" ht="27">
+    <row r="5" ht="28.5" spans="1:19">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1446,7 +2036,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" spans="1:19" ht="27">
+    <row r="6" ht="28.5" spans="1:19">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -1497,7 +2087,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" spans="1:19" ht="27">
+    <row r="7" ht="28.5" spans="1:19">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -1548,7 +2138,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" spans="1:19" ht="27">
+    <row r="8" ht="28.5" spans="1:19">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -1599,7 +2189,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" spans="1:19" ht="27">
+    <row r="9" ht="28.5" spans="1:19">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1650,7 +2240,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19" ht="27">
+    <row r="10" spans="1:19">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -1701,7 +2291,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" spans="1:19" ht="27">
+    <row r="11" ht="28.5" spans="1:19">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1752,7 +2342,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" spans="1:19" ht="54">
+    <row r="12" ht="57" spans="1:19">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -1801,7 +2391,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" spans="1:19" ht="40.5">
+    <row r="13" ht="42.75" spans="1:19">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1843,7 +2433,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" spans="1:19" ht="40.5">
+    <row r="14" ht="28.5" spans="1:19">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -1894,7 +2484,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" spans="1:19" ht="27">
+    <row r="15" ht="28.5" spans="1:19">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1926,9 +2516,9 @@
       <c r="K15" s="7">
         <v>46197</v>
       </c>
-      <c r="L15" s="7" t="str">
+      <c r="L15" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46203</v>
       </c>
       <c r="M15" s="6" t="s">
         <v>39</v>
@@ -1938,12 +2528,14 @@
         <f>IF(AND($C15="Exercise",$K15&lt;&gt;"",$M15&lt;&gt;""),$K15+VLOOKUP($M15,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46199</v>
       </c>
-      <c r="P15" s="7"/>
+      <c r="P15" s="7">
+        <v>46203</v>
+      </c>
       <c r="Q15" s="6"/>
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" spans="1:19" ht="27">
+    <row r="16" ht="28.5" spans="1:19">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -1992,7 +2584,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" spans="1:19" ht="40.5">
+    <row r="17" ht="28.5" spans="1:19">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2021,23 +2613,27 @@
         <v>83</v>
       </c>
       <c r="J17" s="6"/>
-      <c r="K17" s="7"/>
+      <c r="K17" s="7">
+        <v>46203</v>
+      </c>
       <c r="L17" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M17" s="6"/>
+      <c r="M17" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N17" s="6"/>
-      <c r="O17" s="7" t="str">
+      <c r="O17" s="7">
         <f>IF(AND($C17="Exercise",$K17&lt;&gt;"",$M17&lt;&gt;""),$K17+VLOOKUP($M17,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46205</v>
       </c>
       <c r="P17" s="7"/>
       <c r="Q17" s="6"/>
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" spans="1:19" ht="40.5">
+    <row r="18" ht="28.5" spans="1:19">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2082,7 +2678,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" spans="1:19" ht="27">
+    <row r="19" ht="28.5" spans="1:19">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2127,7 +2723,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" spans="1:19" ht="27">
+    <row r="20" ht="28.5" spans="1:19">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2172,7 +2768,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" spans="1:19" ht="67.5">
+    <row r="21" ht="57" spans="1:19">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2217,7 +2813,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" spans="1:19" ht="40.5">
+    <row r="22" ht="42.75" spans="1:19">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2258,7 +2854,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" spans="1:19" ht="40.5">
+    <row r="23" ht="42.75" spans="1:19">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2299,7 +2895,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" spans="1:19" ht="40.5">
+    <row r="24" ht="28.5" spans="1:19">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2344,7 +2940,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" spans="1:19" ht="27">
+    <row r="25" ht="28.5" spans="1:19">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2389,7 +2985,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" spans="1:19" ht="27">
+    <row r="26" ht="28.5" spans="1:19">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -2434,7 +3030,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" spans="1:19" ht="40.5">
+    <row r="27" ht="28.5" spans="1:19">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2479,7 +3075,7 @@
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" spans="1:19" ht="40.5">
+    <row r="28" ht="42.75" spans="1:19">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -2524,7 +3120,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" spans="1:19" ht="54">
+    <row r="29" ht="42.75" spans="1:19">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -2565,7 +3161,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" spans="1:19" ht="40.5">
+    <row r="30" ht="28.5" spans="1:19">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -2606,7 +3202,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" spans="1:19" ht="40.5">
+    <row r="31" ht="28.5" spans="1:19">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -2651,7 +3247,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" spans="1:19" ht="40.5">
+    <row r="32" ht="28.5" spans="1:19">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -2696,7 +3292,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" spans="1:19" ht="40.5">
+    <row r="33" ht="28.5" spans="1:19">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -2741,7 +3337,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" spans="1:19" ht="40.5">
+    <row r="34" ht="28.5" spans="1:19">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -2786,7 +3382,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" spans="1:19" ht="40.5">
+    <row r="35" ht="28.5" spans="1:19">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2831,7 +3427,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" spans="1:19" ht="40.5">
+    <row r="36" ht="28.5" spans="1:19">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -2876,7 +3472,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" spans="1:19" ht="40.5">
+    <row r="37" ht="28.5" spans="1:19">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2921,7 +3517,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" spans="1:19" ht="40.5">
+    <row r="38" ht="28.5" spans="1:19">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -2966,7 +3562,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" spans="1:19" ht="40.5">
+    <row r="39" ht="28.5" spans="1:19">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3011,7 +3607,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" spans="1:19" ht="40.5">
+    <row r="40" ht="28.5" spans="1:19">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3056,7 +3652,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" spans="1:19" ht="54">
+    <row r="41" ht="42.75" spans="1:19">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3101,7 +3697,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" spans="1:19" ht="54">
+    <row r="42" ht="42.75" spans="1:19">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3142,7 +3738,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" spans="1:19" ht="40.5">
+    <row r="43" ht="42.75" spans="1:19">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3183,7 +3779,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" spans="1:19" ht="40.5">
+    <row r="44" ht="28.5" spans="1:19">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3228,7 +3824,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" spans="1:19" ht="40.5">
+    <row r="45" ht="28.5" spans="1:19">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3273,7 +3869,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" spans="1:19" ht="40.5">
+    <row r="46" ht="28.5" spans="1:19">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3318,7 +3914,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" spans="1:19" ht="40.5">
+    <row r="47" ht="28.5" spans="1:19">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3363,7 +3959,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" spans="1:19" ht="40.5">
+    <row r="48" ht="28.5" spans="1:19">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3408,7 +4004,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" spans="1:19" ht="40.5">
+    <row r="49" ht="28.5" spans="1:19">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -3453,7 +4049,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" spans="1:19" ht="40.5">
+    <row r="50" ht="28.5" spans="1:19">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -3498,7 +4094,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" spans="1:19" ht="40.5">
+    <row r="51" ht="28.5" spans="1:19">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -3543,7 +4139,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" spans="1:19" ht="40.5">
+    <row r="52" ht="28.5" spans="1:19">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -3588,7 +4184,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" spans="1:19" ht="40.5">
+    <row r="53" ht="28.5" spans="1:19">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -3633,7 +4229,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" spans="1:19" ht="40.5">
+    <row r="54" ht="28.5" spans="1:19">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -3678,7 +4274,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" spans="1:19" ht="40.5">
+    <row r="55" ht="28.5" spans="1:19">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -3723,7 +4319,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" spans="1:19" ht="54">
+    <row r="56" ht="42.75" spans="1:19">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -3768,7 +4364,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" spans="1:19" ht="67.5">
+    <row r="57" ht="57" spans="1:19">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -3809,7 +4405,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" spans="1:19" ht="40.5">
+    <row r="58" ht="28.5" spans="1:19">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -3854,7 +4450,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" spans="1:19" ht="27">
+    <row r="59" ht="28.5" spans="1:19">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -3899,7 +4495,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" spans="1:19" ht="27">
+    <row r="60" ht="28.5" spans="1:19">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -3944,7 +4540,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" spans="1:19" ht="27">
+    <row r="61" ht="28.5" spans="1:19">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -3989,7 +4585,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" spans="1:19" ht="27">
+    <row r="62" ht="28.5" spans="1:19">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4034,7 +4630,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" spans="1:19" ht="54">
+    <row r="63" ht="42.75" spans="1:19">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4075,7 +4671,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" spans="1:19" ht="54">
+    <row r="64" ht="57" spans="1:19">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4117,35 +4713,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="M2:M64">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="Q2:R64">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4153,21 +4749,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="27">
+    <row r="1" ht="30" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="27">
+    <row r="2" ht="28.5" spans="1:2">
       <c r="A2" s="3" t="s">
         <v>238</v>
       </c>
@@ -4179,7 +4776,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" ht="15" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>240</v>
       </c>
@@ -4188,7 +4785,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" ht="15" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>241</v>
       </c>
@@ -4197,7 +4794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" ht="15" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>242</v>
       </c>
@@ -4206,7 +4803,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" ht="15" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>243</v>
       </c>
@@ -4215,7 +4812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" ht="15" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>244</v>
       </c>
@@ -4224,16 +4821,16 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="27">
+    <row r="9" ht="15" spans="1:2">
       <c r="A9" s="5" t="s">
         <v>245</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="27">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="15" spans="1:2">
       <c r="A10" s="5" t="s">
         <v>246</v>
       </c>
@@ -4246,7 +4843,7 @@
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" ht="15" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>247</v>
       </c>
@@ -4255,7 +4852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" ht="15" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -4264,7 +4861,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" ht="15" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -4273,20 +4870,20 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" ht="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" spans="1:2" ht="27">
+    <row r="17" ht="15" spans="1:2">
       <c r="A17" s="5" t="s">
         <v>248</v>
       </c>
@@ -4294,7 +4891,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" ht="15" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>250</v>
       </c>
@@ -4303,15 +4900,16 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4319,7 +4917,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27">
+    <row r="1" ht="15" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -4389,7 +4987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>263</v>
       </c>
@@ -4401,8 +4999,8 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7 Ex 42
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28245" windowHeight="12465"/>
+    <workbookView windowWidth="19935" windowHeight="7785"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="267">
   <si>
     <t>Order</t>
   </si>
@@ -280,6 +280,9 @@
   </si>
   <si>
     <t>Exercise 34 attempted</t>
+  </si>
+  <si>
+    <t>cantor distribution</t>
   </si>
   <si>
     <t>Do Exercise 41: bounded differences and variance condition.</t>
@@ -821,9 +824,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
@@ -855,14 +858,37 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -877,12 +903,81 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -898,99 +993,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
@@ -1025,7 +1028,127 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1037,13 +1160,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1055,157 +1202,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1224,21 +1227,6 @@
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1290,17 +1278,6 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
@@ -1316,16 +1293,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1334,133 +1337,133 @@
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2567,9 +2570,9 @@
       <c r="K16" s="7">
         <v>46201</v>
       </c>
-      <c r="L16" s="7" t="str">
+      <c r="L16" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46204</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>55</v>
@@ -2579,7 +2582,9 @@
         <f>IF(AND($C16="Exercise",$K16&lt;&gt;"",$M16&lt;&gt;""),$K16+VLOOKUP($M16,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46203</v>
       </c>
-      <c r="P16" s="7"/>
+      <c r="P16" s="7">
+        <v>46204</v>
+      </c>
       <c r="Q16" s="6"/>
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
@@ -2616,9 +2621,9 @@
       <c r="K17" s="7">
         <v>46203</v>
       </c>
-      <c r="L17" s="7" t="str">
+      <c r="L17" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46206</v>
       </c>
       <c r="M17" s="6" t="s">
         <v>30</v>
@@ -2628,7 +2633,9 @@
         <f>IF(AND($C17="Exercise",$K17&lt;&gt;"",$M17&lt;&gt;""),$K17+VLOOKUP($M17,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46205</v>
       </c>
-      <c r="P17" s="7"/>
+      <c r="P17" s="7">
+        <v>46206</v>
+      </c>
       <c r="Q17" s="6"/>
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
@@ -2662,16 +2669,22 @@
         <v>87</v>
       </c>
       <c r="J18" s="6"/>
-      <c r="K18" s="7"/>
+      <c r="K18" s="7">
+        <v>46204</v>
+      </c>
       <c r="L18" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="7" t="str">
+      <c r="M18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="O18" s="7">
         <f>IF(AND($C18="Exercise",$K18&lt;&gt;"",$M18&lt;&gt;""),$K18+VLOOKUP($M18,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46206</v>
       </c>
       <c r="P18" s="7"/>
       <c r="Q18" s="6"/>
@@ -2695,28 +2708,32 @@
         <v>32</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>74</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J19" s="6"/>
-      <c r="K19" s="7"/>
+      <c r="K19" s="7">
+        <v>46205</v>
+      </c>
       <c r="L19" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M19" s="6"/>
+      <c r="M19" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N19" s="6"/>
-      <c r="O19" s="7" t="str">
+      <c r="O19" s="7">
         <f>IF(AND($C19="Exercise",$K19&lt;&gt;"",$M19&lt;&gt;""),$K19+VLOOKUP($M19,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46207</v>
       </c>
       <c r="P19" s="7"/>
       <c r="Q19" s="6"/>
@@ -2740,28 +2757,32 @@
         <v>32</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J20" s="6"/>
-      <c r="K20" s="7"/>
+      <c r="K20" s="7">
+        <v>46206</v>
+      </c>
       <c r="L20" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M20" s="6"/>
+      <c r="M20" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N20" s="6"/>
-      <c r="O20" s="7" t="str">
+      <c r="O20" s="7">
         <f>IF(AND($C20="Exercise",$K20&lt;&gt;"",$M20&lt;&gt;""),$K20+VLOOKUP($M20,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46208</v>
       </c>
       <c r="P20" s="7"/>
       <c r="Q20" s="6"/>
@@ -2785,17 +2806,17 @@
         <v>32</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K21" s="7"/>
       <c r="L21" s="7" t="str">
@@ -2824,18 +2845,18 @@
         <v>19</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="I22" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J22" s="6"/>
       <c r="K22" s="7"/>
@@ -2865,18 +2886,18 @@
         <v>19</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J23" s="6"/>
       <c r="K23" s="7"/>
@@ -2906,22 +2927,22 @@
         <v>6</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F24" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="I24" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="J24" s="6"/>
       <c r="K24" s="7"/>
@@ -2951,22 +2972,22 @@
         <v>6</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J25" s="6"/>
       <c r="K25" s="7"/>
@@ -2996,22 +3017,22 @@
         <v>6</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J26" s="6"/>
       <c r="K26" s="7"/>
@@ -3041,22 +3062,22 @@
         <v>6</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J27" s="6"/>
       <c r="K27" s="7"/>
@@ -3086,23 +3107,23 @@
         <v>60</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K28" s="7"/>
       <c r="L28" s="7" t="str">
@@ -3131,18 +3152,18 @@
         <v>19</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>73</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
       <c r="I29" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J29" s="6"/>
       <c r="K29" s="7"/>
@@ -3172,18 +3193,18 @@
         <v>19</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
       <c r="I30" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J30" s="6"/>
       <c r="K30" s="7"/>
@@ -3213,22 +3234,22 @@
         <v>6</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J31" s="6"/>
       <c r="K31" s="7"/>
@@ -3258,22 +3279,22 @@
         <v>6</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F32" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="I32" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="J32" s="6"/>
       <c r="K32" s="7"/>
@@ -3303,22 +3324,22 @@
         <v>6</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J33" s="6"/>
       <c r="K33" s="7"/>
@@ -3348,22 +3369,22 @@
         <v>6</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J34" s="6"/>
       <c r="K34" s="7"/>
@@ -3393,22 +3414,22 @@
         <v>6</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J35" s="6"/>
       <c r="K35" s="7"/>
@@ -3438,22 +3459,22 @@
         <v>6</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J36" s="6"/>
       <c r="K36" s="7"/>
@@ -3483,22 +3504,22 @@
         <v>6</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J37" s="6"/>
       <c r="K37" s="7"/>
@@ -3528,22 +3549,22 @@
         <v>6</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J38" s="6"/>
       <c r="K38" s="7"/>
@@ -3573,22 +3594,22 @@
         <v>6</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J39" s="6"/>
       <c r="K39" s="7"/>
@@ -3618,22 +3639,22 @@
         <v>6</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J40" s="6"/>
       <c r="K40" s="7"/>
@@ -3663,23 +3684,23 @@
         <v>60</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G41" s="6"/>
       <c r="H41" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K41" s="7"/>
       <c r="L41" s="7" t="str">
@@ -3708,18 +3729,18 @@
         <v>19</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
       <c r="I42" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J42" s="6"/>
       <c r="K42" s="7"/>
@@ -3749,18 +3770,18 @@
         <v>19</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
       <c r="I43" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J43" s="6"/>
       <c r="K43" s="7"/>
@@ -3790,22 +3811,22 @@
         <v>6</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J44" s="6"/>
       <c r="K44" s="7"/>
@@ -3835,22 +3856,22 @@
         <v>6</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F45" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="I45" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>175</v>
       </c>
       <c r="J45" s="6"/>
       <c r="K45" s="7"/>
@@ -3880,22 +3901,22 @@
         <v>6</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J46" s="6"/>
       <c r="K46" s="7"/>
@@ -3925,22 +3946,22 @@
         <v>6</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J47" s="6"/>
       <c r="K47" s="7"/>
@@ -3970,22 +3991,22 @@
         <v>6</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J48" s="6"/>
       <c r="K48" s="7"/>
@@ -4015,22 +4036,22 @@
         <v>6</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J49" s="6"/>
       <c r="K49" s="7"/>
@@ -4060,22 +4081,22 @@
         <v>6</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J50" s="6"/>
       <c r="K50" s="7"/>
@@ -4105,22 +4126,22 @@
         <v>6</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J51" s="6"/>
       <c r="K51" s="7"/>
@@ -4150,22 +4171,22 @@
         <v>6</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J52" s="6"/>
       <c r="K52" s="7"/>
@@ -4195,22 +4216,22 @@
         <v>6</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J53" s="6"/>
       <c r="K53" s="7"/>
@@ -4240,22 +4261,22 @@
         <v>6</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J54" s="6"/>
       <c r="K54" s="7"/>
@@ -4285,22 +4306,22 @@
         <v>6</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J55" s="6"/>
       <c r="K55" s="7"/>
@@ -4330,23 +4351,23 @@
         <v>60</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G56" s="6"/>
       <c r="H56" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K56" s="7"/>
       <c r="L56" s="7" t="str">
@@ -4375,18 +4396,18 @@
         <v>19</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J57" s="6"/>
       <c r="K57" s="7"/>
@@ -4416,22 +4437,22 @@
         <v>6</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58" s="7"/>
@@ -4461,22 +4482,22 @@
         <v>6</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F59" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>218</v>
-      </c>
-      <c r="G59" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="H59" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="I59" s="6" t="s">
-        <v>217</v>
       </c>
       <c r="J59" s="6"/>
       <c r="K59" s="7"/>
@@ -4506,22 +4527,22 @@
         <v>6</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J60" s="6"/>
       <c r="K60" s="7"/>
@@ -4551,22 +4572,22 @@
         <v>6</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J61" s="6"/>
       <c r="K61" s="7"/>
@@ -4596,22 +4617,22 @@
         <v>6</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J62" s="6"/>
       <c r="K62" s="7"/>
@@ -4638,21 +4659,21 @@
         <v>46238</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
       <c r="I63" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="J63" s="6"/>
       <c r="K63" s="7"/>
@@ -4679,21 +4700,21 @@
         <v>46239</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
       <c r="I64" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J64" s="6"/>
       <c r="K64" s="7"/>
@@ -4760,16 +4781,16 @@
   <sheetData>
     <row r="1" ht="30" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="28.5" spans="1:2">
       <c r="A2" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -4778,7 +4799,7 @@
     </row>
     <row r="4" ht="15" spans="1:2">
       <c r="A4" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B4" s="4">
         <f>COUNTA('Master Schedule'!$A$2:$A$64)</f>
@@ -4787,7 +4808,7 @@
     </row>
     <row r="5" ht="15" spans="1:2">
       <c r="A5" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B5" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Read")</f>
@@ -4796,7 +4817,7 @@
     </row>
     <row r="6" ht="15" spans="1:2">
       <c r="A6" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Exercise")</f>
@@ -4805,7 +4826,7 @@
     </row>
     <row r="7" ht="15" spans="1:2">
       <c r="A7" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Gate")</f>
@@ -4814,7 +4835,7 @@
     </row>
     <row r="8" ht="15" spans="1:2">
       <c r="A8" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Summary")</f>
@@ -4823,20 +4844,20 @@
     </row>
     <row r="9" ht="15" spans="1:2">
       <c r="A9" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" ht="15" spans="1:2">
       <c r="A10" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4845,7 +4866,7 @@
     </row>
     <row r="12" ht="15" spans="1:2">
       <c r="A12" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Totally ignorance")</f>
@@ -4858,7 +4879,7 @@
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Spark")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="15" spans="1:2">
@@ -4867,7 +4888,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" ht="15" spans="1:2">
@@ -4876,7 +4897,7 @@
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -4885,18 +4906,18 @@
     </row>
     <row r="17" ht="15" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" ht="15" spans="1:2">
       <c r="A18" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -4922,24 +4943,24 @@
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -4950,10 +4971,10 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
@@ -4964,10 +4985,10 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D4" s="2">
         <v>2</v>
@@ -4978,10 +4999,10 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C5" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
@@ -4989,13 +5010,13 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chap7, Ex 18, 31, 32
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19935" windowHeight="7785"/>
+    <workbookView windowWidth="19935" windowHeight="7935"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="267">
   <si>
     <t>Order</t>
   </si>
@@ -824,11 +824,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -850,8 +850,24 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -865,23 +881,8 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -894,61 +895,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -971,6 +926,44 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -978,8 +971,15 @@
     </font>
     <font>
       <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -995,7 +995,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1028,13 +1028,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1046,19 +1058,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1070,61 +1082,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1148,13 +1106,85 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1166,37 +1196,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1208,7 +1208,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1219,15 +1219,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1242,21 +1233,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1279,8 +1255,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1289,18 +1265,31 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
+      <top/>
       <bottom style="double">
-        <color theme="4"/>
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1319,151 +1308,162 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2672,9 +2672,9 @@
       <c r="K18" s="7">
         <v>46204</v>
       </c>
-      <c r="L18" s="7" t="str">
+      <c r="L18" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46206</v>
       </c>
       <c r="M18" s="6" t="s">
         <v>55</v>
@@ -2686,7 +2686,9 @@
         <f>IF(AND($C18="Exercise",$K18&lt;&gt;"",$M18&lt;&gt;""),$K18+VLOOKUP($M18,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46206</v>
       </c>
-      <c r="P18" s="7"/>
+      <c r="P18" s="7">
+        <v>46206</v>
+      </c>
       <c r="Q18" s="6"/>
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
@@ -2723,9 +2725,9 @@
       <c r="K19" s="7">
         <v>46205</v>
       </c>
-      <c r="L19" s="7" t="str">
+      <c r="L19" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46208</v>
       </c>
       <c r="M19" s="6" t="s">
         <v>39</v>
@@ -2735,7 +2737,9 @@
         <f>IF(AND($C19="Exercise",$K19&lt;&gt;"",$M19&lt;&gt;""),$K19+VLOOKUP($M19,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46207</v>
       </c>
-      <c r="P19" s="7"/>
+      <c r="P19" s="7">
+        <v>46208</v>
+      </c>
       <c r="Q19" s="6"/>
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
@@ -2818,10 +2822,11 @@
       <c r="J21" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="K21" s="7">
+        <v>46207</v>
+      </c>
+      <c r="L21" s="7">
+        <v>46207</v>
       </c>
       <c r="M21" s="6"/>
       <c r="N21" s="6"/>
@@ -2859,10 +2864,11 @@
         <v>102</v>
       </c>
       <c r="J22" s="6"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="K22" s="7">
+        <v>46208</v>
+      </c>
+      <c r="L22" s="7">
+        <v>46208</v>
       </c>
       <c r="M22" s="6"/>
       <c r="N22" s="6"/>
@@ -2900,10 +2906,11 @@
         <v>105</v>
       </c>
       <c r="J23" s="6"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="K23" s="7">
+        <v>46209</v>
+      </c>
+      <c r="L23" s="7">
+        <v>46209</v>
       </c>
       <c r="M23" s="6"/>
       <c r="N23" s="6"/>
@@ -2945,16 +2952,20 @@
         <v>105</v>
       </c>
       <c r="J24" s="6"/>
-      <c r="K24" s="7"/>
+      <c r="K24" s="7">
+        <v>46210</v>
+      </c>
       <c r="L24" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M24" s="6"/>
+      <c r="M24" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N24" s="6"/>
-      <c r="O24" s="7" t="str">
+      <c r="O24" s="7">
         <f>IF(AND($C24="Exercise",$K24&lt;&gt;"",$M24&lt;&gt;""),$K24+VLOOKUP($M24,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46212</v>
       </c>
       <c r="P24" s="7"/>
       <c r="Q24" s="6"/>
@@ -2990,16 +3001,20 @@
         <v>112</v>
       </c>
       <c r="J25" s="6"/>
-      <c r="K25" s="7"/>
+      <c r="K25" s="7">
+        <v>46210</v>
+      </c>
       <c r="L25" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M25" s="6"/>
+      <c r="M25" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N25" s="6"/>
-      <c r="O25" s="7" t="str">
+      <c r="O25" s="7">
         <f>IF(AND($C25="Exercise",$K25&lt;&gt;"",$M25&lt;&gt;""),$K25+VLOOKUP($M25,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46212</v>
       </c>
       <c r="P25" s="7"/>
       <c r="Q25" s="6"/>
@@ -3035,16 +3050,20 @@
         <v>116</v>
       </c>
       <c r="J26" s="6"/>
-      <c r="K26" s="7"/>
+      <c r="K26" s="7">
+        <v>46211</v>
+      </c>
       <c r="L26" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M26" s="6"/>
+      <c r="M26" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="N26" s="6"/>
-      <c r="O26" s="7" t="str">
+      <c r="O26" s="7">
         <f>IF(AND($C26="Exercise",$K26&lt;&gt;"",$M26&lt;&gt;""),$K26+VLOOKUP($M26,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46213</v>
       </c>
       <c r="P26" s="7"/>
       <c r="Q26" s="6"/>
@@ -4848,7 +4867,7 @@
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" ht="15" spans="1:2">
@@ -4857,7 +4876,7 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4879,7 +4898,7 @@
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Spark")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" ht="15" spans="1:2">
@@ -4897,7 +4916,7 @@
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:2">

</xml_diff>

<commit_message>
Chap 7, Ex 32, 40
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,22 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_7DE5626199A21D5814B1DB7DF443FB989E2099A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70A07018-4AEB-4D65-AEC2-493488269AED}"/>
   <bookViews>
-    <workbookView windowWidth="19935" windowHeight="7935"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="267">
   <si>
     <t>Order</t>
   </si>
@@ -822,15 +842,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -850,158 +866,17 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="9"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1026,194 +901,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1221,332 +910,59 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
+      <font>
+        <b/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1560,24 +976,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1587,43 +986,54 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" name="Order"/>
-    <tableColumn id="2" name="Planned Date"/>
-    <tableColumn id="3" name="Task Type"/>
-    <tableColumn id="4" name="Phase"/>
-    <tableColumn id="5" name="Section(s)"/>
-    <tableColumn id="6" name="Task"/>
-    <tableColumn id="7" name="Exercise"/>
-    <tableColumn id="8" name="Related Result / Reason"/>
-    <tableColumn id="9" name="Prerequisite"/>
-    <tableColumn id="10" name="Proceed Gate"/>
-    <tableColumn id="11" name="Actual Start"/>
-    <tableColumn id="12" name="Actual End"/>
-    <tableColumn id="13" name="First-pass Status"/>
-    <tableColumn id="14" name="Key Blocker"/>
-    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
-    <tableColumn id="16" name="Redo Result"/>
-    <tableColumn id="17" name="Proceed?"/>
-    <tableColumn id="18" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
+      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
+      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" name="First-pass Status"/>
-    <tableColumn id="2" name="Meaning"/>
-    <tableColumn id="3" name="Recommended Action"/>
-    <tableColumn id="4" name="Redo Offset Days"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1772,14 +1182,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1801,7 +1211,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:19">
+    <row r="1" spans="1:19" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1860,7 +1270,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="42.75" spans="1:19">
+    <row r="2" spans="1:19" ht="54">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1901,7 +1311,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" ht="42.75" spans="1:19">
+    <row r="3" spans="1:19" ht="54">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1942,7 +1352,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" ht="28.5" spans="1:19">
+    <row r="4" spans="1:19" ht="27">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1988,7 +1398,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" ht="28.5" spans="1:19">
+    <row r="5" spans="1:19" ht="27">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2039,7 +1449,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" ht="28.5" spans="1:19">
+    <row r="6" spans="1:19" ht="27">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2090,7 +1500,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" ht="28.5" spans="1:19">
+    <row r="7" spans="1:19" ht="27">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2141,7 +1551,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" ht="28.5" spans="1:19">
+    <row r="8" spans="1:19" ht="27">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2192,7 +1602,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" ht="28.5" spans="1:19">
+    <row r="9" spans="1:19" ht="27">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2243,7 +1653,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" ht="27">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2294,7 +1704,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" ht="28.5" spans="1:19">
+    <row r="11" spans="1:19" ht="27">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2345,7 +1755,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" ht="57" spans="1:19">
+    <row r="12" spans="1:19" ht="54">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2394,7 +1804,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" ht="42.75" spans="1:19">
+    <row r="13" spans="1:19" ht="40.5">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2436,7 +1846,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" ht="28.5" spans="1:19">
+    <row r="14" spans="1:19" ht="40.5">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2487,7 +1897,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" ht="28.5" spans="1:19">
+    <row r="15" spans="1:19" ht="27">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2538,7 +1948,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" ht="28.5" spans="1:19">
+    <row r="16" spans="1:19" ht="27">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2589,7 +1999,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" ht="28.5" spans="1:19">
+    <row r="17" spans="1:19" ht="40.5">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2640,7 +2050,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" ht="28.5" spans="1:19">
+    <row r="18" spans="1:19" ht="40.5">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2693,7 +2103,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" ht="28.5" spans="1:19">
+    <row r="19" spans="1:19" ht="27">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2744,7 +2154,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" ht="28.5" spans="1:19">
+    <row r="20" spans="1:19" ht="27">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2793,7 +2203,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" ht="57" spans="1:19">
+    <row r="21" spans="1:19" ht="67.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2839,7 +2249,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" ht="42.75" spans="1:19">
+    <row r="22" spans="1:19" ht="40.5">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2881,7 +2291,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" ht="42.75" spans="1:19">
+    <row r="23" spans="1:19" ht="40.5">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2923,7 +2333,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" ht="28.5" spans="1:19">
+    <row r="24" spans="1:19" ht="40.5">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2972,7 +2382,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" ht="28.5" spans="1:19">
+    <row r="25" spans="1:19" ht="27">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -3021,7 +2431,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" ht="28.5" spans="1:19">
+    <row r="26" spans="1:19" ht="27">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -3070,7 +2480,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" ht="28.5" spans="1:19">
+    <row r="27" spans="1:19" ht="40.5">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -3099,23 +2509,27 @@
         <v>120</v>
       </c>
       <c r="J27" s="6"/>
-      <c r="K27" s="7"/>
+      <c r="K27" s="7">
+        <v>46213</v>
+      </c>
       <c r="L27" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M27" s="6"/>
+      <c r="M27" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="N27" s="6"/>
-      <c r="O27" s="7" t="str">
+      <c r="O27" s="7">
         <f>IF(AND($C27="Exercise",$K27&lt;&gt;"",$M27&lt;&gt;""),$K27+VLOOKUP($M27,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46215</v>
       </c>
       <c r="P27" s="7"/>
       <c r="Q27" s="6"/>
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" ht="42.75" spans="1:19">
+    <row r="28" spans="1:19" ht="40.5">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -3160,7 +2574,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" ht="42.75" spans="1:19">
+    <row r="29" spans="1:19" ht="54">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3201,7 +2615,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" ht="28.5" spans="1:19">
+    <row r="30" spans="1:19" ht="40.5">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3242,7 +2656,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" ht="28.5" spans="1:19">
+    <row r="31" spans="1:19" ht="40.5">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3287,7 +2701,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" ht="28.5" spans="1:19">
+    <row r="32" spans="1:19" ht="40.5">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -3332,7 +2746,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" ht="28.5" spans="1:19">
+    <row r="33" spans="1:19" ht="40.5">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3377,7 +2791,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" ht="28.5" spans="1:19">
+    <row r="34" spans="1:19" ht="40.5">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -3422,7 +2836,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" ht="28.5" spans="1:19">
+    <row r="35" spans="1:19" ht="40.5">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3467,7 +2881,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" ht="28.5" spans="1:19">
+    <row r="36" spans="1:19" ht="40.5">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -3512,7 +2926,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" ht="28.5" spans="1:19">
+    <row r="37" spans="1:19" ht="40.5">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3557,7 +2971,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" ht="28.5" spans="1:19">
+    <row r="38" spans="1:19" ht="40.5">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3602,7 +3016,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" ht="28.5" spans="1:19">
+    <row r="39" spans="1:19" ht="40.5">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3647,7 +3061,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" ht="28.5" spans="1:19">
+    <row r="40" spans="1:19" ht="40.5">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3692,7 +3106,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" ht="42.75" spans="1:19">
+    <row r="41" spans="1:19" ht="54">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3737,7 +3151,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" ht="42.75" spans="1:19">
+    <row r="42" spans="1:19" ht="54">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3778,7 +3192,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" ht="42.75" spans="1:19">
+    <row r="43" spans="1:19" ht="40.5">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3819,7 +3233,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" ht="28.5" spans="1:19">
+    <row r="44" spans="1:19" ht="40.5">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3864,7 +3278,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" ht="28.5" spans="1:19">
+    <row r="45" spans="1:19" ht="40.5">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3909,7 +3323,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" ht="28.5" spans="1:19">
+    <row r="46" spans="1:19" ht="40.5">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3954,7 +3368,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" ht="28.5" spans="1:19">
+    <row r="47" spans="1:19" ht="40.5">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3999,7 +3413,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" ht="28.5" spans="1:19">
+    <row r="48" spans="1:19" ht="40.5">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -4044,7 +3458,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" ht="28.5" spans="1:19">
+    <row r="49" spans="1:19" ht="40.5">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -4089,7 +3503,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" ht="28.5" spans="1:19">
+    <row r="50" spans="1:19" ht="40.5">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -4134,7 +3548,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" ht="28.5" spans="1:19">
+    <row r="51" spans="1:19" ht="40.5">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -4179,7 +3593,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" ht="28.5" spans="1:19">
+    <row r="52" spans="1:19" ht="40.5">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -4224,7 +3638,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" ht="28.5" spans="1:19">
+    <row r="53" spans="1:19" ht="40.5">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -4269,7 +3683,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" ht="28.5" spans="1:19">
+    <row r="54" spans="1:19" ht="40.5">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -4314,7 +3728,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" ht="28.5" spans="1:19">
+    <row r="55" spans="1:19" ht="40.5">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -4359,7 +3773,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" ht="42.75" spans="1:19">
+    <row r="56" spans="1:19" ht="54">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -4404,7 +3818,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" ht="57" spans="1:19">
+    <row r="57" spans="1:19" ht="67.5">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -4445,7 +3859,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" ht="28.5" spans="1:19">
+    <row r="58" spans="1:19" ht="40.5">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4490,7 +3904,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" ht="28.5" spans="1:19">
+    <row r="59" spans="1:19" ht="27">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4535,7 +3949,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" ht="28.5" spans="1:19">
+    <row r="60" spans="1:19" ht="27">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4580,7 +3994,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" ht="28.5" spans="1:19">
+    <row r="61" spans="1:19" ht="27">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4625,7 +4039,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" ht="28.5" spans="1:19">
+    <row r="62" spans="1:19" ht="27">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4670,7 +4084,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" ht="42.75" spans="1:19">
+    <row r="63" spans="1:19" ht="54">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4711,7 +4125,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" ht="57" spans="1:19">
+    <row r="64" spans="1:19" ht="54">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4753,35 +4167,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64">
+    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64">
+    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4789,22 +4203,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" spans="1:2">
+    <row r="1" spans="1:2" ht="27">
       <c r="A1" s="1" t="s">
         <v>238</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" ht="28.5" spans="1:2">
+    <row r="2" spans="1:2" ht="27">
       <c r="A2" s="3" t="s">
         <v>239</v>
       </c>
@@ -4816,7 +4229,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" ht="15" spans="1:2">
+    <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>241</v>
       </c>
@@ -4825,7 +4238,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="15" spans="1:2">
+    <row r="5" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>242</v>
       </c>
@@ -4834,7 +4247,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="15" spans="1:2">
+    <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>243</v>
       </c>
@@ -4843,7 +4256,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" ht="15" spans="1:2">
+    <row r="7" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>244</v>
       </c>
@@ -4852,7 +4265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="15" spans="1:2">
+    <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>245</v>
       </c>
@@ -4861,7 +4274,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15" spans="1:2">
+    <row r="9" spans="1:2" ht="27">
       <c r="A9" s="5" t="s">
         <v>246</v>
       </c>
@@ -4870,20 +4283,20 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" ht="15" spans="1:2">
+    <row r="10" spans="1:2" ht="27">
       <c r="A10" s="5" t="s">
         <v>247</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" ht="15" spans="1:2">
+    <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>248</v>
       </c>
@@ -4892,16 +4305,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="15" spans="1:2">
+    <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Spark")</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" ht="15" spans="1:2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -4910,7 +4323,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" ht="15" spans="1:2">
+    <row r="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
@@ -4923,7 +4336,7 @@
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" ht="15" spans="1:2">
+    <row r="17" spans="1:2" ht="27">
       <c r="A17" s="5" t="s">
         <v>249</v>
       </c>
@@ -4931,7 +4344,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="18" ht="15" spans="1:2">
+    <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>251</v>
       </c>
@@ -4940,16 +4353,15 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4957,7 +4369,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:4">
+    <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -5027,7 +4439,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>264</v>
       </c>
@@ -5039,8 +4451,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, Ex 8,9
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_7DE5626199A21D5814B1DB7DF443FB989E2099A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0518A86D-D530-420C-9C05-2F227003E132}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_4DAF32EFFC52D7E756F74D2D611117399016891C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27E53138-3F3F-45DA-9FC3-8B11783F46D3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="267">
   <si>
     <t>Order</t>
   </si>
@@ -844,7 +844,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -933,7 +933,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -991,10 +991,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2517,9 +2513,9 @@
       <c r="K27" s="7">
         <v>46213</v>
       </c>
-      <c r="L27" s="7" t="str">
+      <c r="L27" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46215</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>55</v>
@@ -2529,7 +2525,9 @@
         <f>IF(AND($C27="Exercise",$K27&lt;&gt;"",$M27&lt;&gt;""),$K27+VLOOKUP($M27,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46215</v>
       </c>
-      <c r="P27" s="7"/>
+      <c r="P27" s="7">
+        <v>46215</v>
+      </c>
       <c r="Q27" s="6"/>
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
@@ -2605,10 +2603,11 @@
         <v>127</v>
       </c>
       <c r="J29" s="6"/>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="K29" s="7">
+        <v>46216</v>
+      </c>
+      <c r="L29" s="7">
+        <v>46217</v>
       </c>
       <c r="M29" s="6"/>
       <c r="N29" s="6"/>
@@ -2646,10 +2645,11 @@
         <v>130</v>
       </c>
       <c r="J30" s="6"/>
-      <c r="K30" s="7"/>
-      <c r="L30" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="K30" s="7">
+        <v>46218</v>
+      </c>
+      <c r="L30" s="7">
+        <v>46220</v>
       </c>
       <c r="M30" s="6"/>
       <c r="N30" s="6"/>
@@ -2691,16 +2691,20 @@
         <v>135</v>
       </c>
       <c r="J31" s="6"/>
-      <c r="K31" s="7"/>
+      <c r="K31" s="7">
+        <v>46221</v>
+      </c>
       <c r="L31" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M31" s="6"/>
+      <c r="M31" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N31" s="6"/>
-      <c r="O31" s="7" t="str">
+      <c r="O31" s="7">
         <f>IF(AND($C31="Exercise",$K31&lt;&gt;"",$M31&lt;&gt;""),$K31+VLOOKUP($M31,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46223</v>
       </c>
       <c r="P31" s="7"/>
       <c r="Q31" s="6"/>
@@ -4286,7 +4290,7 @@
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="27">
@@ -4326,7 +4330,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:2">

</xml_diff>

<commit_message>
Chap 7, Ex 10
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,42 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_4DAF32EFFC52D7E756F74D2D611117399016891C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27E53138-3F3F-45DA-9FC3-8B11783F46D3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="19935" windowHeight="7935"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="267">
   <si>
     <t>Order</t>
   </si>
@@ -842,11 +822,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -867,16 +851,157 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Carlito"/>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -901,8 +1026,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -910,52 +1221,339 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+  <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <font>
-        <b/>
-      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -969,14 +1567,17 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFE699"/>
+          <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="1"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -986,50 +1587,43 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
-      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
-      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
+    <tableColumn id="1" name="Order"/>
+    <tableColumn id="2" name="Planned Date"/>
+    <tableColumn id="3" name="Task Type"/>
+    <tableColumn id="4" name="Phase"/>
+    <tableColumn id="5" name="Section(s)"/>
+    <tableColumn id="6" name="Task"/>
+    <tableColumn id="7" name="Exercise"/>
+    <tableColumn id="8" name="Related Result / Reason"/>
+    <tableColumn id="9" name="Prerequisite"/>
+    <tableColumn id="10" name="Proceed Gate"/>
+    <tableColumn id="11" name="Actual Start"/>
+    <tableColumn id="12" name="Actual End"/>
+    <tableColumn id="13" name="First-pass Status"/>
+    <tableColumn id="14" name="Key Blocker"/>
+    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
+    <tableColumn id="16" name="Redo Result"/>
+    <tableColumn id="17" name="Proceed?"/>
+    <tableColumn id="18" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
+    <tableColumn id="1" name="First-pass Status"/>
+    <tableColumn id="2" name="Meaning"/>
+    <tableColumn id="3" name="Recommended Action"/>
+    <tableColumn id="4" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1178,14 +1772,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1207,7 +1801,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="32.1" customHeight="1">
+    <row r="1" ht="32.1" customHeight="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1266,7 +1860,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="54">
+    <row r="2" ht="42.75" spans="1:19">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1307,7 +1901,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" spans="1:19" ht="54">
+    <row r="3" ht="42.75" spans="1:19">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1348,7 +1942,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" spans="1:19" ht="27">
+    <row r="4" ht="28.5" spans="1:19">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1394,7 +1988,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" spans="1:19" ht="27">
+    <row r="5" ht="28.5" spans="1:19">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1445,7 +2039,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" spans="1:19" ht="27">
+    <row r="6" ht="28.5" spans="1:19">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -1496,7 +2090,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" spans="1:19" ht="27">
+    <row r="7" ht="28.5" spans="1:19">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -1547,7 +2141,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" spans="1:19" ht="27">
+    <row r="8" ht="28.5" spans="1:19">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -1598,7 +2192,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" spans="1:19" ht="27">
+    <row r="9" ht="28.5" spans="1:19">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1649,7 +2243,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19" ht="27">
+    <row r="10" spans="1:19">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -1700,7 +2294,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" spans="1:19" ht="27">
+    <row r="11" ht="28.5" spans="1:19">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1751,7 +2345,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" spans="1:19" ht="54">
+    <row r="12" ht="57" spans="1:19">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -1800,7 +2394,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" spans="1:19" ht="40.5">
+    <row r="13" ht="42.75" spans="1:19">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1842,7 +2436,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" spans="1:19" ht="40.5">
+    <row r="14" ht="28.5" spans="1:19">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -1893,7 +2487,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" spans="1:19" ht="27">
+    <row r="15" ht="28.5" spans="1:19">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1944,7 +2538,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" spans="1:19" ht="27">
+    <row r="16" ht="28.5" spans="1:19">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -1995,7 +2589,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" spans="1:19" ht="40.5">
+    <row r="17" ht="28.5" spans="1:19">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2046,7 +2640,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" spans="1:19" ht="40.5">
+    <row r="18" ht="28.5" spans="1:19">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2099,7 +2693,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" spans="1:19" ht="27">
+    <row r="19" ht="28.5" spans="1:19">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2150,7 +2744,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" spans="1:19" ht="27">
+    <row r="20" ht="28.5" spans="1:19">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2201,7 +2795,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" spans="1:19" ht="67.5">
+    <row r="21" ht="57" spans="1:19">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2247,7 +2841,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" spans="1:19" ht="40.5">
+    <row r="22" ht="42.75" spans="1:19">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2289,7 +2883,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" spans="1:19" ht="40.5">
+    <row r="23" ht="42.75" spans="1:19">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2331,7 +2925,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" spans="1:19" ht="40.5">
+    <row r="24" ht="28.5" spans="1:19">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2374,12 +2968,14 @@
         <f>IF(AND($C24="Exercise",$K24&lt;&gt;"",$M24&lt;&gt;""),$K24+VLOOKUP($M24,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46212</v>
       </c>
-      <c r="P24" s="7"/>
+      <c r="P24" s="7">
+        <v>46212</v>
+      </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" spans="1:19" ht="27">
+    <row r="25" ht="28.5" spans="1:19">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2430,7 +3026,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" spans="1:19" ht="27">
+    <row r="26" ht="28.5" spans="1:19">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -2481,7 +3077,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" spans="1:19" ht="40.5">
+    <row r="27" ht="28.5" spans="1:19">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2532,7 +3128,7 @@
       <c r="R27" s="6"/>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" spans="1:19" ht="40.5">
+    <row r="28" ht="42.75" spans="1:19">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -2578,7 +3174,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" spans="1:19" ht="54">
+    <row r="29" ht="42.75" spans="1:19">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -2620,7 +3216,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" spans="1:19" ht="40.5">
+    <row r="30" ht="28.5" spans="1:19">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -2662,7 +3258,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" spans="1:19" ht="40.5">
+    <row r="31" ht="28.5" spans="1:19">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -2694,9 +3290,9 @@
       <c r="K31" s="7">
         <v>46221</v>
       </c>
-      <c r="L31" s="7" t="str">
+      <c r="L31" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46223</v>
       </c>
       <c r="M31" s="6" t="s">
         <v>39</v>
@@ -2706,12 +3302,14 @@
         <f>IF(AND($C31="Exercise",$K31&lt;&gt;"",$M31&lt;&gt;""),$K31+VLOOKUP($M31,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46223</v>
       </c>
-      <c r="P31" s="7"/>
+      <c r="P31" s="7">
+        <v>46223</v>
+      </c>
       <c r="Q31" s="6"/>
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" spans="1:19" ht="40.5">
+    <row r="32" ht="28.5" spans="1:19">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -2740,23 +3338,27 @@
         <v>135</v>
       </c>
       <c r="J32" s="6"/>
-      <c r="K32" s="7"/>
+      <c r="K32" s="7">
+        <v>46222</v>
+      </c>
       <c r="L32" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M32" s="6"/>
+      <c r="M32" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N32" s="6"/>
-      <c r="O32" s="7" t="str">
+      <c r="O32" s="7">
         <f>IF(AND($C32="Exercise",$K32&lt;&gt;"",$M32&lt;&gt;""),$K32+VLOOKUP($M32,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46224</v>
       </c>
       <c r="P32" s="7"/>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" spans="1:19" ht="40.5">
+    <row r="33" ht="28.5" spans="1:19">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -2785,23 +3387,27 @@
         <v>135</v>
       </c>
       <c r="J33" s="6"/>
-      <c r="K33" s="7"/>
+      <c r="K33" s="7">
+        <v>46223</v>
+      </c>
       <c r="L33" s="7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="M33" s="6"/>
+      <c r="M33" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N33" s="6"/>
-      <c r="O33" s="7" t="str">
+      <c r="O33" s="7">
         <f>IF(AND($C33="Exercise",$K33&lt;&gt;"",$M33&lt;&gt;""),$K33+VLOOKUP($M33,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46225</v>
       </c>
       <c r="P33" s="7"/>
       <c r="Q33" s="6"/>
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" spans="1:19" ht="40.5">
+    <row r="34" ht="28.5" spans="1:19">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -2846,7 +3452,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" spans="1:19" ht="40.5">
+    <row r="35" ht="28.5" spans="1:19">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2891,7 +3497,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" spans="1:19" ht="40.5">
+    <row r="36" ht="28.5" spans="1:19">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -2936,7 +3542,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" spans="1:19" ht="40.5">
+    <row r="37" ht="28.5" spans="1:19">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2981,7 +3587,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" spans="1:19" ht="40.5">
+    <row r="38" ht="28.5" spans="1:19">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3026,7 +3632,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" spans="1:19" ht="40.5">
+    <row r="39" ht="28.5" spans="1:19">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3071,7 +3677,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" spans="1:19" ht="40.5">
+    <row r="40" ht="28.5" spans="1:19">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3116,7 +3722,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" spans="1:19" ht="54">
+    <row r="41" ht="42.75" spans="1:19">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3161,7 +3767,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" spans="1:19" ht="54">
+    <row r="42" ht="42.75" spans="1:19">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3202,7 +3808,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" spans="1:19" ht="40.5">
+    <row r="43" ht="42.75" spans="1:19">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3243,7 +3849,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" spans="1:19" ht="40.5">
+    <row r="44" ht="28.5" spans="1:19">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3288,7 +3894,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" spans="1:19" ht="40.5">
+    <row r="45" ht="28.5" spans="1:19">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3333,7 +3939,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" spans="1:19" ht="40.5">
+    <row r="46" ht="28.5" spans="1:19">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3378,7 +3984,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" spans="1:19" ht="40.5">
+    <row r="47" ht="28.5" spans="1:19">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3423,7 +4029,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" spans="1:19" ht="40.5">
+    <row r="48" ht="28.5" spans="1:19">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3468,7 +4074,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" spans="1:19" ht="40.5">
+    <row r="49" ht="28.5" spans="1:19">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -3513,7 +4119,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" spans="1:19" ht="40.5">
+    <row r="50" ht="28.5" spans="1:19">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -3558,7 +4164,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" spans="1:19" ht="40.5">
+    <row r="51" ht="28.5" spans="1:19">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -3603,7 +4209,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" spans="1:19" ht="40.5">
+    <row r="52" ht="28.5" spans="1:19">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -3648,7 +4254,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" spans="1:19" ht="40.5">
+    <row r="53" ht="28.5" spans="1:19">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -3693,7 +4299,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" spans="1:19" ht="40.5">
+    <row r="54" ht="28.5" spans="1:19">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -3738,7 +4344,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" spans="1:19" ht="40.5">
+    <row r="55" ht="28.5" spans="1:19">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -3783,7 +4389,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" spans="1:19" ht="54">
+    <row r="56" ht="42.75" spans="1:19">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -3828,7 +4434,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" spans="1:19" ht="67.5">
+    <row r="57" ht="57" spans="1:19">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -3869,7 +4475,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" spans="1:19" ht="40.5">
+    <row r="58" ht="28.5" spans="1:19">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -3914,7 +4520,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" spans="1:19" ht="27">
+    <row r="59" ht="28.5" spans="1:19">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -3959,7 +4565,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" spans="1:19" ht="27">
+    <row r="60" ht="28.5" spans="1:19">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4004,7 +4610,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" spans="1:19" ht="27">
+    <row r="61" ht="28.5" spans="1:19">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4049,7 +4655,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" spans="1:19" ht="27">
+    <row r="62" ht="28.5" spans="1:19">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4094,7 +4700,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" spans="1:19" ht="54">
+    <row r="63" ht="42.75" spans="1:19">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4135,7 +4741,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" spans="1:19" ht="54">
+    <row r="64" ht="57" spans="1:19">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4177,35 +4783,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="M2:M64">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="Q2:R64">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4213,21 +4819,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="27">
+    <row r="1" ht="30" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>238</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="27">
+    <row r="2" ht="28.5" spans="1:2">
       <c r="A2" s="3" t="s">
         <v>239</v>
       </c>
@@ -4239,7 +4846,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" ht="15" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>241</v>
       </c>
@@ -4248,7 +4855,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" ht="15" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>242</v>
       </c>
@@ -4257,7 +4864,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" ht="15" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>243</v>
       </c>
@@ -4266,7 +4873,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" ht="15" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>244</v>
       </c>
@@ -4275,7 +4882,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" ht="15" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>245</v>
       </c>
@@ -4284,29 +4891,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="27">
+    <row r="9" ht="15" spans="1:2">
       <c r="A9" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="27">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" ht="15" spans="1:2">
       <c r="A10" s="5" t="s">
         <v>247</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" ht="15" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>248</v>
       </c>
@@ -4315,7 +4922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" ht="15" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -4324,16 +4931,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" ht="15" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" ht="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
@@ -4346,7 +4953,7 @@
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" spans="1:2" ht="27">
+    <row r="17" ht="15" spans="1:2">
       <c r="A17" s="5" t="s">
         <v>249</v>
       </c>
@@ -4354,7 +4961,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" ht="15" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>251</v>
       </c>
@@ -4363,15 +4970,16 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4379,7 +4987,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27">
+    <row r="1" ht="15" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -4449,7 +5057,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>264</v>
       </c>
@@ -4461,8 +5069,8 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, Ex 12
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="267">
   <si>
     <t>Order</t>
   </si>
@@ -824,8 +824,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
@@ -853,22 +853,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -887,14 +871,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -909,7 +893,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
@@ -919,21 +917,6 @@
     <font>
       <b/>
       <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -972,8 +955,32 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -989,13 +996,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1028,7 +1028,103 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1040,19 +1136,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1064,43 +1178,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1112,103 +1202,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1222,36 +1222,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -1272,6 +1246,26 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -1283,6 +1277,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1310,160 +1319,151 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3436,16 +3436,20 @@
         <v>135</v>
       </c>
       <c r="J34" s="6"/>
-      <c r="K34" s="7"/>
+      <c r="K34" s="7">
+        <v>46224</v>
+      </c>
       <c r="L34" s="7" t="str">
         <f t="shared" ref="L34:L64" si="1">IF($P34&lt;&gt;"",$P34,"")</f>
         <v/>
       </c>
-      <c r="M34" s="6"/>
+      <c r="M34" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="N34" s="6"/>
-      <c r="O34" s="7" t="str">
+      <c r="O34" s="7">
         <f>IF(AND($C34="Exercise",$K34&lt;&gt;"",$M34&lt;&gt;""),$K34+VLOOKUP($M34,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46226</v>
       </c>
       <c r="P34" s="7"/>
       <c r="Q34" s="6"/>
@@ -4803,11 +4807,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
+    <dataValidation type="list" sqref="Q2:R64">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
     <dataValidation type="list" sqref="M2:M64">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64">
-      <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4906,7 +4910,7 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4928,7 +4932,7 @@
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Spark")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" ht="15" spans="1:2">

</xml_diff>

<commit_message>
Chap 7, Ex 16
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19935" windowHeight="7935"/>
+    <workbookView windowWidth="28245" windowHeight="12615"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="268">
   <si>
     <t>Order</t>
   </si>
@@ -379,6 +379,9 @@
   </si>
   <si>
     <t>Exercise 32 attempted</t>
+  </si>
+  <si>
+    <t>2026-7-20 redo2</t>
   </si>
   <si>
     <t>Proceed gate: can you explain why Kronecker lemma is not just algebra but a device for SLLN?</t>
@@ -826,8 +829,8 @@
   <numFmts count="5">
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="23">
@@ -851,21 +854,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -879,33 +867,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -926,6 +899,44 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -933,7 +944,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -954,17 +973,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -986,18 +996,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1028,7 +1031,139 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1040,55 +1175,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1100,103 +1199,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1208,7 +1211,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1219,32 +1222,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1275,8 +1252,32 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1296,174 +1297,176 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color theme="4"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="35" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="27" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3125,7 +3128,9 @@
         <v>46215</v>
       </c>
       <c r="Q27" s="6"/>
-      <c r="R27" s="6"/>
+      <c r="R27" s="6" t="s">
+        <v>121</v>
+      </c>
       <c r="S27" s="4"/>
     </row>
     <row r="28" ht="42.75" spans="1:19">
@@ -3145,17 +3150,17 @@
         <v>36</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K28" s="7">
         <v>46215</v>
@@ -3185,18 +3190,18 @@
         <v>19</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>73</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
       <c r="I29" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J29" s="6"/>
       <c r="K29" s="7">
@@ -3227,18 +3232,18 @@
         <v>19</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
       <c r="I30" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J30" s="6"/>
       <c r="K30" s="7">
@@ -3269,22 +3274,22 @@
         <v>6</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J31" s="6"/>
       <c r="K31" s="7">
@@ -3320,30 +3325,30 @@
         <v>6</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F32" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="I32" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>135</v>
       </c>
       <c r="J32" s="6"/>
       <c r="K32" s="7">
         <v>46222</v>
       </c>
-      <c r="L32" s="7" t="str">
+      <c r="L32" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46224</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>39</v>
@@ -3353,7 +3358,9 @@
         <f>IF(AND($C32="Exercise",$K32&lt;&gt;"",$M32&lt;&gt;""),$K32+VLOOKUP($M32,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46224</v>
       </c>
-      <c r="P32" s="7"/>
+      <c r="P32" s="7">
+        <v>46224</v>
+      </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
@@ -3369,22 +3376,22 @@
         <v>6</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J33" s="6"/>
       <c r="K33" s="7">
@@ -3418,22 +3425,22 @@
         <v>6</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J34" s="6"/>
       <c r="K34" s="7">
@@ -3467,34 +3474,38 @@
         <v>6</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J35" s="6"/>
-      <c r="K35" s="7"/>
+      <c r="K35" s="7">
+        <v>46225</v>
+      </c>
       <c r="L35" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M35" s="6"/>
+      <c r="M35" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N35" s="6"/>
-      <c r="O35" s="7" t="str">
+      <c r="O35" s="7">
         <f>IF(AND($C35="Exercise",$K35&lt;&gt;"",$M35&lt;&gt;""),$K35+VLOOKUP($M35,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46227</v>
       </c>
       <c r="P35" s="7"/>
       <c r="Q35" s="6"/>
@@ -3512,22 +3523,22 @@
         <v>6</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J36" s="6"/>
       <c r="K36" s="7"/>
@@ -3557,22 +3568,22 @@
         <v>6</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J37" s="6"/>
       <c r="K37" s="7"/>
@@ -3602,22 +3613,22 @@
         <v>6</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J38" s="6"/>
       <c r="K38" s="7"/>
@@ -3647,22 +3658,22 @@
         <v>6</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J39" s="6"/>
       <c r="K39" s="7"/>
@@ -3692,22 +3703,22 @@
         <v>6</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J40" s="6"/>
       <c r="K40" s="7"/>
@@ -3737,23 +3748,23 @@
         <v>60</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G41" s="6"/>
       <c r="H41" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K41" s="7"/>
       <c r="L41" s="7" t="str">
@@ -3782,18 +3793,18 @@
         <v>19</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
       <c r="I42" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J42" s="6"/>
       <c r="K42" s="7"/>
@@ -3823,18 +3834,18 @@
         <v>19</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
       <c r="I43" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J43" s="6"/>
       <c r="K43" s="7"/>
@@ -3864,22 +3875,22 @@
         <v>6</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J44" s="6"/>
       <c r="K44" s="7"/>
@@ -3909,22 +3920,22 @@
         <v>6</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F45" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="I45" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>176</v>
       </c>
       <c r="J45" s="6"/>
       <c r="K45" s="7"/>
@@ -3954,22 +3965,22 @@
         <v>6</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J46" s="6"/>
       <c r="K46" s="7"/>
@@ -3999,22 +4010,22 @@
         <v>6</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J47" s="6"/>
       <c r="K47" s="7"/>
@@ -4044,22 +4055,22 @@
         <v>6</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J48" s="6"/>
       <c r="K48" s="7"/>
@@ -4089,22 +4100,22 @@
         <v>6</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J49" s="6"/>
       <c r="K49" s="7"/>
@@ -4134,22 +4145,22 @@
         <v>6</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J50" s="6"/>
       <c r="K50" s="7"/>
@@ -4179,22 +4190,22 @@
         <v>6</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J51" s="6"/>
       <c r="K51" s="7"/>
@@ -4224,22 +4235,22 @@
         <v>6</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J52" s="6"/>
       <c r="K52" s="7"/>
@@ -4269,22 +4280,22 @@
         <v>6</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J53" s="6"/>
       <c r="K53" s="7"/>
@@ -4314,22 +4325,22 @@
         <v>6</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J54" s="6"/>
       <c r="K54" s="7"/>
@@ -4359,22 +4370,22 @@
         <v>6</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J55" s="6"/>
       <c r="K55" s="7"/>
@@ -4404,23 +4415,23 @@
         <v>60</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G56" s="6"/>
       <c r="H56" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K56" s="7"/>
       <c r="L56" s="7" t="str">
@@ -4449,18 +4460,18 @@
         <v>19</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J57" s="6"/>
       <c r="K57" s="7"/>
@@ -4490,22 +4501,22 @@
         <v>6</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58" s="7"/>
@@ -4535,22 +4546,22 @@
         <v>6</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F59" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>219</v>
-      </c>
-      <c r="G59" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="H59" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="I59" s="6" t="s">
-        <v>218</v>
       </c>
       <c r="J59" s="6"/>
       <c r="K59" s="7"/>
@@ -4580,22 +4591,22 @@
         <v>6</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J60" s="6"/>
       <c r="K60" s="7"/>
@@ -4625,22 +4636,22 @@
         <v>6</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J61" s="6"/>
       <c r="K61" s="7"/>
@@ -4670,22 +4681,22 @@
         <v>6</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J62" s="6"/>
       <c r="K62" s="7"/>
@@ -4712,21 +4723,21 @@
         <v>46238</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
       <c r="I63" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="J63" s="6"/>
       <c r="K63" s="7"/>
@@ -4753,21 +4764,21 @@
         <v>46239</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
       <c r="I64" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J64" s="6"/>
       <c r="K64" s="7"/>
@@ -4807,11 +4818,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
+    <dataValidation type="list" sqref="M2:M64">
+      <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
+    </dataValidation>
     <dataValidation type="list" sqref="Q2:R64">
       <formula1>"Y,N"</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="M2:M64">
-      <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4834,16 +4845,16 @@
   <sheetData>
     <row r="1" ht="30" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="28.5" spans="1:2">
       <c r="A2" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -4852,7 +4863,7 @@
     </row>
     <row r="4" ht="15" spans="1:2">
       <c r="A4" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B4" s="4">
         <f>COUNTA('Master Schedule'!$A$2:$A$64)</f>
@@ -4861,7 +4872,7 @@
     </row>
     <row r="5" ht="15" spans="1:2">
       <c r="A5" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B5" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Read")</f>
@@ -4870,7 +4881,7 @@
     </row>
     <row r="6" ht="15" spans="1:2">
       <c r="A6" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Exercise")</f>
@@ -4879,7 +4890,7 @@
     </row>
     <row r="7" ht="15" spans="1:2">
       <c r="A7" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Gate")</f>
@@ -4888,7 +4899,7 @@
     </row>
     <row r="8" ht="15" spans="1:2">
       <c r="A8" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Summary")</f>
@@ -4897,20 +4908,20 @@
     </row>
     <row r="9" ht="15" spans="1:2">
       <c r="A9" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" ht="15" spans="1:2">
       <c r="A10" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4919,7 +4930,7 @@
     </row>
     <row r="12" ht="15" spans="1:2">
       <c r="A12" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Totally ignorance")</f>
@@ -4941,7 +4952,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" ht="15" spans="1:2">
@@ -4959,18 +4970,18 @@
     </row>
     <row r="17" ht="15" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" ht="15" spans="1:2">
       <c r="A18" s="5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -4996,24 +5007,24 @@
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -5024,10 +5035,10 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
@@ -5038,10 +5049,10 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D4" s="2">
         <v>2</v>
@@ -5052,10 +5063,10 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
@@ -5063,13 +5074,13 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chap 7, Ex 35
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,17 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_4145FF17F15E472E9283AFDC7933D76ADA4E604E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{451E8275-973A-46F8-A47A-47840C60D51E}"/>
   <bookViews>
-    <workbookView windowWidth="28245" windowHeight="12615"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -825,15 +845,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -854,157 +870,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
+      <sz val="9"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1029,194 +904,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1224,332 +913,59 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="28" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
+      <font>
+        <b/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1563,24 +979,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1590,43 +989,50 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" name="Order"/>
-    <tableColumn id="2" name="Planned Date"/>
-    <tableColumn id="3" name="Task Type"/>
-    <tableColumn id="4" name="Phase"/>
-    <tableColumn id="5" name="Section(s)"/>
-    <tableColumn id="6" name="Task"/>
-    <tableColumn id="7" name="Exercise"/>
-    <tableColumn id="8" name="Related Result / Reason"/>
-    <tableColumn id="9" name="Prerequisite"/>
-    <tableColumn id="10" name="Proceed Gate"/>
-    <tableColumn id="11" name="Actual Start"/>
-    <tableColumn id="12" name="Actual End"/>
-    <tableColumn id="13" name="First-pass Status"/>
-    <tableColumn id="14" name="Key Blocker"/>
-    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
-    <tableColumn id="16" name="Redo Result"/>
-    <tableColumn id="17" name="Proceed?"/>
-    <tableColumn id="18" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
+      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
+      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" name="First-pass Status"/>
-    <tableColumn id="2" name="Meaning"/>
-    <tableColumn id="3" name="Recommended Action"/>
-    <tableColumn id="4" name="Redo Offset Days"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1775,14 +1181,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1804,7 +1210,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:19">
+    <row r="1" spans="1:19" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1863,7 +1269,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="42.75" spans="1:19">
+    <row r="2" spans="1:19" ht="54">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1904,7 +1310,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" ht="42.75" spans="1:19">
+    <row r="3" spans="1:19" ht="54">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1945,7 +1351,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" ht="28.5" spans="1:19">
+    <row r="4" spans="1:19" ht="27">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1991,7 +1397,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" ht="28.5" spans="1:19">
+    <row r="5" spans="1:19" ht="27">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2042,7 +1448,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" ht="28.5" spans="1:19">
+    <row r="6" spans="1:19" ht="27">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2093,7 +1499,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" ht="28.5" spans="1:19">
+    <row r="7" spans="1:19" ht="27">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2144,7 +1550,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" ht="28.5" spans="1:19">
+    <row r="8" spans="1:19" ht="27">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2195,7 +1601,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" ht="28.5" spans="1:19">
+    <row r="9" spans="1:19" ht="27">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2246,7 +1652,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" ht="27">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2297,7 +1703,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" ht="28.5" spans="1:19">
+    <row r="11" spans="1:19" ht="27">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2348,7 +1754,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" ht="57" spans="1:19">
+    <row r="12" spans="1:19" ht="54">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2397,7 +1803,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" ht="42.75" spans="1:19">
+    <row r="13" spans="1:19" ht="40.5">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2439,7 +1845,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" ht="28.5" spans="1:19">
+    <row r="14" spans="1:19" ht="40.5">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2490,7 +1896,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" ht="28.5" spans="1:19">
+    <row r="15" spans="1:19" ht="27">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2541,7 +1947,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" ht="28.5" spans="1:19">
+    <row r="16" spans="1:19" ht="27">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2592,7 +1998,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" ht="28.5" spans="1:19">
+    <row r="17" spans="1:19" ht="40.5">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2643,7 +2049,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" ht="28.5" spans="1:19">
+    <row r="18" spans="1:19" ht="40.5">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2696,7 +2102,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" ht="28.5" spans="1:19">
+    <row r="19" spans="1:19" ht="27">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2747,7 +2153,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" ht="28.5" spans="1:19">
+    <row r="20" spans="1:19" ht="27">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2798,7 +2204,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" ht="57" spans="1:19">
+    <row r="21" spans="1:19" ht="67.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2844,7 +2250,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" ht="42.75" spans="1:19">
+    <row r="22" spans="1:19" ht="40.5">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2886,7 +2292,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" ht="42.75" spans="1:19">
+    <row r="23" spans="1:19" ht="40.5">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2928,7 +2334,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" ht="28.5" spans="1:19">
+    <row r="24" spans="1:19" ht="40.5">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2978,7 +2384,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" ht="28.5" spans="1:19">
+    <row r="25" spans="1:19" ht="27">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -3029,7 +2435,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" ht="28.5" spans="1:19">
+    <row r="26" spans="1:19" ht="27">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -3080,7 +2486,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" ht="28.5" spans="1:19">
+    <row r="27" spans="1:19" ht="40.5">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -3133,7 +2539,7 @@
       </c>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" ht="42.75" spans="1:19">
+    <row r="28" spans="1:19" ht="40.5">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -3179,7 +2585,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" ht="42.75" spans="1:19">
+    <row r="29" spans="1:19" ht="54">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3221,7 +2627,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" ht="28.5" spans="1:19">
+    <row r="30" spans="1:19" ht="40.5">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3263,7 +2669,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" ht="28.5" spans="1:19">
+    <row r="31" spans="1:19" ht="40.5">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3314,7 +2720,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" ht="28.5" spans="1:19">
+    <row r="32" spans="1:19" ht="40.5">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -3365,7 +2771,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" ht="28.5" spans="1:19">
+    <row r="33" spans="1:19" ht="40.5">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3397,9 +2803,9 @@
       <c r="K33" s="7">
         <v>46223</v>
       </c>
-      <c r="L33" s="7" t="str">
+      <c r="L33" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>46225</v>
       </c>
       <c r="M33" s="6" t="s">
         <v>39</v>
@@ -3409,12 +2815,14 @@
         <f>IF(AND($C33="Exercise",$K33&lt;&gt;"",$M33&lt;&gt;""),$K33+VLOOKUP($M33,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46225</v>
       </c>
-      <c r="P33" s="7"/>
+      <c r="P33" s="7">
+        <v>46225</v>
+      </c>
       <c r="Q33" s="6"/>
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" ht="28.5" spans="1:19">
+    <row r="34" spans="1:19" ht="40.5">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -3463,7 +2871,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" ht="28.5" spans="1:19">
+    <row r="35" spans="1:19" ht="40.5">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3512,7 +2920,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" ht="28.5" spans="1:19">
+    <row r="36" spans="1:19" ht="40.5">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -3557,7 +2965,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" ht="28.5" spans="1:19">
+    <row r="37" spans="1:19" ht="40.5">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3602,7 +3010,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" ht="28.5" spans="1:19">
+    <row r="38" spans="1:19" ht="40.5">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3647,7 +3055,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" ht="28.5" spans="1:19">
+    <row r="39" spans="1:19" ht="40.5">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3692,7 +3100,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" ht="28.5" spans="1:19">
+    <row r="40" spans="1:19" ht="40.5">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3737,7 +3145,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" ht="42.75" spans="1:19">
+    <row r="41" spans="1:19" ht="54">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3782,7 +3190,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" ht="42.75" spans="1:19">
+    <row r="42" spans="1:19" ht="54">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3823,7 +3231,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" ht="42.75" spans="1:19">
+    <row r="43" spans="1:19" ht="40.5">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3864,7 +3272,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" ht="28.5" spans="1:19">
+    <row r="44" spans="1:19" ht="40.5">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3909,7 +3317,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" ht="28.5" spans="1:19">
+    <row r="45" spans="1:19" ht="40.5">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3954,7 +3362,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" ht="28.5" spans="1:19">
+    <row r="46" spans="1:19" ht="40.5">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3999,7 +3407,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" ht="28.5" spans="1:19">
+    <row r="47" spans="1:19" ht="40.5">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -4044,7 +3452,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" ht="28.5" spans="1:19">
+    <row r="48" spans="1:19" ht="40.5">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -4089,7 +3497,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" ht="28.5" spans="1:19">
+    <row r="49" spans="1:19" ht="40.5">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -4134,7 +3542,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" ht="28.5" spans="1:19">
+    <row r="50" spans="1:19" ht="40.5">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -4179,7 +3587,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" ht="28.5" spans="1:19">
+    <row r="51" spans="1:19" ht="40.5">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -4224,7 +3632,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" ht="28.5" spans="1:19">
+    <row r="52" spans="1:19" ht="40.5">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -4269,7 +3677,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" ht="28.5" spans="1:19">
+    <row r="53" spans="1:19" ht="40.5">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -4314,7 +3722,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" ht="28.5" spans="1:19">
+    <row r="54" spans="1:19" ht="40.5">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -4359,7 +3767,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" ht="28.5" spans="1:19">
+    <row r="55" spans="1:19" ht="40.5">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -4404,7 +3812,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" ht="42.75" spans="1:19">
+    <row r="56" spans="1:19" ht="54">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -4449,7 +3857,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" ht="57" spans="1:19">
+    <row r="57" spans="1:19" ht="67.5">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -4490,7 +3898,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" ht="28.5" spans="1:19">
+    <row r="58" spans="1:19" ht="40.5">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4535,7 +3943,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" ht="28.5" spans="1:19">
+    <row r="59" spans="1:19" ht="27">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4580,7 +3988,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" ht="28.5" spans="1:19">
+    <row r="60" spans="1:19" ht="27">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4625,7 +4033,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" ht="28.5" spans="1:19">
+    <row r="61" spans="1:19" ht="27">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4670,7 +4078,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" ht="28.5" spans="1:19">
+    <row r="62" spans="1:19" ht="27">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4715,7 +4123,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" ht="42.75" spans="1:19">
+    <row r="63" spans="1:19" ht="54">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4756,7 +4164,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" ht="57" spans="1:19">
+    <row r="64" spans="1:19" ht="54">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4798,35 +4206,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64">
+    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64">
+    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4834,22 +4242,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" spans="1:2">
+    <row r="1" spans="1:2" ht="27">
       <c r="A1" s="1" t="s">
         <v>239</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" ht="28.5" spans="1:2">
+    <row r="2" spans="1:2" ht="27">
       <c r="A2" s="3" t="s">
         <v>240</v>
       </c>
@@ -4861,7 +4268,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" ht="15" spans="1:2">
+    <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>242</v>
       </c>
@@ -4870,7 +4277,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="15" spans="1:2">
+    <row r="5" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>243</v>
       </c>
@@ -4879,7 +4286,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="15" spans="1:2">
+    <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>244</v>
       </c>
@@ -4888,7 +4295,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" ht="15" spans="1:2">
+    <row r="7" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>245</v>
       </c>
@@ -4897,7 +4304,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="15" spans="1:2">
+    <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>246</v>
       </c>
@@ -4906,29 +4313,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15" spans="1:2">
+    <row r="9" spans="1:2" ht="27">
       <c r="A9" s="5" t="s">
         <v>247</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" ht="15" spans="1:2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="27">
       <c r="A10" s="5" t="s">
         <v>248</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" ht="15" spans="1:2">
+    <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>249</v>
       </c>
@@ -4937,7 +4344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="15" spans="1:2">
+    <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -4946,7 +4353,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" ht="15" spans="1:2">
+    <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -4955,7 +4362,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" ht="15" spans="1:2">
+    <row r="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
@@ -4968,7 +4375,7 @@
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" ht="15" spans="1:2">
+    <row r="17" spans="1:2" ht="27">
       <c r="A17" s="5" t="s">
         <v>250</v>
       </c>
@@ -4976,7 +4383,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="18" ht="15" spans="1:2">
+    <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>252</v>
       </c>
@@ -4985,16 +4392,15 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -5002,7 +4408,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:4">
+    <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -5072,7 +4478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>265</v>
       </c>
@@ -5084,8 +4490,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, Ex 35,43
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,42 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_4145FF17F15E472E9283AFDC7933D76ADA4E604E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{451E8275-973A-46F8-A47A-47840C60D51E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="28245" windowHeight="12615"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="268">
   <si>
     <t>Order</t>
   </si>
@@ -845,11 +825,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -870,16 +854,157 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Carlito"/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -904,8 +1029,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -913,52 +1224,339 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+  <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <font>
-        <b/>
-      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -972,14 +1570,17 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFE699"/>
+          <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="1"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -989,50 +1590,43 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
-      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
-      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
+    <tableColumn id="1" name="Order"/>
+    <tableColumn id="2" name="Planned Date"/>
+    <tableColumn id="3" name="Task Type"/>
+    <tableColumn id="4" name="Phase"/>
+    <tableColumn id="5" name="Section(s)"/>
+    <tableColumn id="6" name="Task"/>
+    <tableColumn id="7" name="Exercise"/>
+    <tableColumn id="8" name="Related Result / Reason"/>
+    <tableColumn id="9" name="Prerequisite"/>
+    <tableColumn id="10" name="Proceed Gate"/>
+    <tableColumn id="11" name="Actual Start"/>
+    <tableColumn id="12" name="Actual End"/>
+    <tableColumn id="13" name="First-pass Status"/>
+    <tableColumn id="14" name="Key Blocker"/>
+    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
+    <tableColumn id="16" name="Redo Result"/>
+    <tableColumn id="17" name="Proceed?"/>
+    <tableColumn id="18" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
+    <tableColumn id="1" name="First-pass Status"/>
+    <tableColumn id="2" name="Meaning"/>
+    <tableColumn id="3" name="Recommended Action"/>
+    <tableColumn id="4" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1181,25 +1775,25 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="37.5" customWidth="1"/>
+    <col min="6" max="6" width="37.45" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="19.875" customWidth="1"/>
-    <col min="9" max="9" width="21.75" customWidth="1"/>
-    <col min="10" max="10" width="18.375" customWidth="1"/>
-    <col min="11" max="11" width="17.875" customWidth="1"/>
+    <col min="8" max="8" width="19.9083333333333" customWidth="1"/>
+    <col min="9" max="9" width="21.725" customWidth="1"/>
+    <col min="10" max="10" width="18.3666666666667" customWidth="1"/>
+    <col min="11" max="11" width="17.9083333333333" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
     <col min="14" max="14" width="28" customWidth="1"/>
@@ -1210,7 +1804,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="32.1" customHeight="1">
+    <row r="1" ht="32.15" customHeight="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1269,7 +1863,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="54">
+    <row r="2" ht="42.75" spans="1:19">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1310,7 +1904,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" spans="1:19" ht="54">
+    <row r="3" ht="42.75" spans="1:19">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1351,7 +1945,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" spans="1:19" ht="27">
+    <row r="4" ht="28.5" spans="1:19">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1397,7 +1991,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" spans="1:19" ht="27">
+    <row r="5" ht="28.5" spans="1:19">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1448,7 +2042,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" spans="1:19" ht="27">
+    <row r="6" ht="28.5" spans="1:19">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -1499,7 +2093,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" spans="1:19" ht="27">
+    <row r="7" ht="28.5" spans="1:19">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -1550,7 +2144,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" spans="1:19" ht="27">
+    <row r="8" ht="28.5" spans="1:19">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -1601,7 +2195,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" spans="1:19" ht="27">
+    <row r="9" ht="28.5" spans="1:19">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1652,7 +2246,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19" ht="27">
+    <row r="10" spans="1:19">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -1703,7 +2297,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" spans="1:19" ht="27">
+    <row r="11" ht="28.5" spans="1:19">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1754,7 +2348,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" spans="1:19" ht="54">
+    <row r="12" ht="57" spans="1:19">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -1803,7 +2397,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" spans="1:19" ht="40.5">
+    <row r="13" ht="42.75" spans="1:19">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1845,7 +2439,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" spans="1:19" ht="40.5">
+    <row r="14" ht="28.5" spans="1:19">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -1896,7 +2490,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" spans="1:19" ht="27">
+    <row r="15" ht="28.5" spans="1:19">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1947,7 +2541,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" spans="1:19" ht="27">
+    <row r="16" ht="28.5" spans="1:19">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -1998,7 +2592,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" spans="1:19" ht="40.5">
+    <row r="17" ht="28.5" spans="1:19">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2049,7 +2643,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" spans="1:19" ht="40.5">
+    <row r="18" ht="28.5" spans="1:19">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2102,7 +2696,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" spans="1:19" ht="27">
+    <row r="19" ht="28.5" spans="1:19">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2153,7 +2747,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" spans="1:19" ht="27">
+    <row r="20" ht="28.5" spans="1:19">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2204,7 +2798,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" spans="1:19" ht="67.5">
+    <row r="21" ht="57" spans="1:19">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2250,7 +2844,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" spans="1:19" ht="40.5">
+    <row r="22" ht="42.75" spans="1:19">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2292,7 +2886,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" spans="1:19" ht="40.5">
+    <row r="23" ht="42.75" spans="1:19">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2334,7 +2928,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" spans="1:19" ht="40.5">
+    <row r="24" ht="28.5" spans="1:19">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2384,7 +2978,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" spans="1:19" ht="27">
+    <row r="25" ht="28.5" spans="1:19">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2435,7 +3029,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" spans="1:19" ht="27">
+    <row r="26" ht="28.5" spans="1:19">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -2486,7 +3080,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" spans="1:19" ht="40.5">
+    <row r="27" ht="28.5" spans="1:19">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2539,7 +3133,7 @@
       </c>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" spans="1:19" ht="40.5">
+    <row r="28" ht="42.75" spans="1:19">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -2585,7 +3179,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" spans="1:19" ht="54">
+    <row r="29" ht="42.75" spans="1:19">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -2627,7 +3221,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" spans="1:19" ht="40.5">
+    <row r="30" ht="28.5" spans="1:19">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -2669,7 +3263,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" spans="1:19" ht="40.5">
+    <row r="31" ht="42.75" spans="1:19">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -2720,7 +3314,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" spans="1:19" ht="40.5">
+    <row r="32" ht="42.75" spans="1:19">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -2771,7 +3365,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" spans="1:19" ht="40.5">
+    <row r="33" ht="42.75" spans="1:19">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -2822,7 +3416,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" spans="1:19" ht="40.5">
+    <row r="34" ht="42.75" spans="1:19">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -2854,9 +3448,9 @@
       <c r="K34" s="7">
         <v>46224</v>
       </c>
-      <c r="L34" s="7" t="str">
+      <c r="L34" s="7">
         <f t="shared" ref="L34:L64" si="1">IF($P34&lt;&gt;"",$P34,"")</f>
-        <v/>
+        <v>46226</v>
       </c>
       <c r="M34" s="6" t="s">
         <v>55</v>
@@ -2866,12 +3460,14 @@
         <f>IF(AND($C34="Exercise",$K34&lt;&gt;"",$M34&lt;&gt;""),$K34+VLOOKUP($M34,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46226</v>
       </c>
-      <c r="P34" s="7"/>
+      <c r="P34" s="7">
+        <v>46226</v>
+      </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" spans="1:19" ht="40.5">
+    <row r="35" ht="42.75" spans="1:19">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2903,9 +3499,9 @@
       <c r="K35" s="7">
         <v>46225</v>
       </c>
-      <c r="L35" s="7" t="str">
+      <c r="L35" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46227</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>39</v>
@@ -2915,12 +3511,14 @@
         <f>IF(AND($C35="Exercise",$K35&lt;&gt;"",$M35&lt;&gt;""),$K35+VLOOKUP($M35,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46227</v>
       </c>
-      <c r="P35" s="7"/>
+      <c r="P35" s="7">
+        <v>46227</v>
+      </c>
       <c r="Q35" s="6"/>
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" spans="1:19" ht="40.5">
+    <row r="36" ht="42.75" spans="1:19">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -2949,23 +3547,27 @@
         <v>136</v>
       </c>
       <c r="J36" s="6"/>
-      <c r="K36" s="7"/>
+      <c r="K36" s="7">
+        <v>46226</v>
+      </c>
       <c r="L36" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M36" s="6"/>
+      <c r="M36" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="N36" s="6"/>
-      <c r="O36" s="7" t="str">
+      <c r="O36" s="7">
         <f>IF(AND($C36="Exercise",$K36&lt;&gt;"",$M36&lt;&gt;""),$K36+VLOOKUP($M36,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46228</v>
       </c>
       <c r="P36" s="7"/>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" spans="1:19" ht="40.5">
+    <row r="37" ht="42.75" spans="1:19">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2994,23 +3596,29 @@
         <v>136</v>
       </c>
       <c r="J37" s="6"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7" t="str">
+      <c r="K37" s="7">
+        <v>46227</v>
+      </c>
+      <c r="L37" s="7">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="M37" s="6"/>
+        <v>46231</v>
+      </c>
+      <c r="M37" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N37" s="6"/>
-      <c r="O37" s="7" t="str">
+      <c r="O37" s="7">
         <f>IF(AND($C37="Exercise",$K37&lt;&gt;"",$M37&lt;&gt;""),$K37+VLOOKUP($M37,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="P37" s="7"/>
+        <v>46229</v>
+      </c>
+      <c r="P37" s="7">
+        <v>46231</v>
+      </c>
       <c r="Q37" s="6"/>
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" spans="1:19" ht="40.5">
+    <row r="38" ht="42.75" spans="1:19">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3039,23 +3647,27 @@
         <v>136</v>
       </c>
       <c r="J38" s="6"/>
-      <c r="K38" s="7"/>
+      <c r="K38" s="7">
+        <v>46229</v>
+      </c>
       <c r="L38" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M38" s="6"/>
+      <c r="M38" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N38" s="6"/>
-      <c r="O38" s="7" t="str">
+      <c r="O38" s="7">
         <f>IF(AND($C38="Exercise",$K38&lt;&gt;"",$M38&lt;&gt;""),$K38+VLOOKUP($M38,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46231</v>
       </c>
       <c r="P38" s="7"/>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" spans="1:19" ht="40.5">
+    <row r="39" ht="42.75" spans="1:19">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3100,7 +3712,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" spans="1:19" ht="40.5">
+    <row r="40" ht="42.75" spans="1:19">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3145,7 +3757,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" spans="1:19" ht="54">
+    <row r="41" ht="42.75" spans="1:19">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3190,7 +3802,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" spans="1:19" ht="54">
+    <row r="42" ht="42.75" spans="1:19">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3231,7 +3843,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" spans="1:19" ht="40.5">
+    <row r="43" ht="42.75" spans="1:19">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3272,7 +3884,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" spans="1:19" ht="40.5">
+    <row r="44" ht="42.75" spans="1:19">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3317,7 +3929,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" spans="1:19" ht="40.5">
+    <row r="45" ht="42.75" spans="1:19">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3362,7 +3974,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" spans="1:19" ht="40.5">
+    <row r="46" ht="42.75" spans="1:19">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3407,7 +4019,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" spans="1:19" ht="40.5">
+    <row r="47" ht="42.75" spans="1:19">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3452,7 +4064,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" spans="1:19" ht="40.5">
+    <row r="48" ht="42.75" spans="1:19">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3497,7 +4109,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" spans="1:19" ht="40.5">
+    <row r="49" ht="42.75" spans="1:19">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -3542,7 +4154,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" spans="1:19" ht="40.5">
+    <row r="50" ht="42.75" spans="1:19">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -3587,7 +4199,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" spans="1:19" ht="40.5">
+    <row r="51" ht="42.75" spans="1:19">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -3632,7 +4244,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" spans="1:19" ht="40.5">
+    <row r="52" ht="42.75" spans="1:19">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -3677,7 +4289,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" spans="1:19" ht="40.5">
+    <row r="53" ht="42.75" spans="1:19">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -3722,7 +4334,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" spans="1:19" ht="40.5">
+    <row r="54" ht="42.75" spans="1:19">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -3767,7 +4379,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" spans="1:19" ht="40.5">
+    <row r="55" ht="42.75" spans="1:19">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -3812,7 +4424,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" spans="1:19" ht="54">
+    <row r="56" ht="42.75" spans="1:19">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -3857,7 +4469,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" spans="1:19" ht="67.5">
+    <row r="57" ht="57" spans="1:19">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -3898,7 +4510,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" spans="1:19" ht="40.5">
+    <row r="58" ht="28.5" spans="1:19">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -3943,7 +4555,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" spans="1:19" ht="27">
+    <row r="59" ht="28.5" spans="1:19">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -3988,7 +4600,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" spans="1:19" ht="27">
+    <row r="60" ht="28.5" spans="1:19">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4033,7 +4645,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" spans="1:19" ht="27">
+    <row r="61" ht="28.5" spans="1:19">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4078,7 +4690,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" spans="1:19" ht="27">
+    <row r="62" ht="28.5" spans="1:19">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4123,7 +4735,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" spans="1:19" ht="54">
+    <row r="63" ht="42.75" spans="1:19">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4164,7 +4776,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" spans="1:19" ht="54">
+    <row r="64" ht="57" spans="1:19">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4206,35 +4818,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="M2:M64">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="Q2:R64">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4242,21 +4854,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="27">
+    <row r="1" ht="30" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>239</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="27">
+    <row r="2" ht="28.5" spans="1:2">
       <c r="A2" s="3" t="s">
         <v>240</v>
       </c>
@@ -4268,7 +4881,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" ht="15" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>242</v>
       </c>
@@ -4277,7 +4890,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" ht="15" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>243</v>
       </c>
@@ -4286,7 +4899,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" ht="15" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>244</v>
       </c>
@@ -4295,7 +4908,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" ht="15" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>245</v>
       </c>
@@ -4304,7 +4917,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" ht="15" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>246</v>
       </c>
@@ -4313,29 +4926,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="27">
+    <row r="9" ht="15" spans="1:2">
       <c r="A9" s="5" t="s">
         <v>247</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="27">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" ht="15" spans="1:2">
       <c r="A10" s="5" t="s">
         <v>248</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" ht="15" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>249</v>
       </c>
@@ -4344,38 +4957,38 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" ht="15" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Spark")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" ht="15" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" ht="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" spans="1:2" ht="27">
+    <row r="17" ht="15" spans="1:2">
       <c r="A17" s="5" t="s">
         <v>250</v>
       </c>
@@ -4383,7 +4996,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" ht="15" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>252</v>
       </c>
@@ -4392,15 +5005,16 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4408,7 +5022,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27">
+    <row r="1" ht="15" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -4478,7 +5092,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>265</v>
       </c>
@@ -4490,8 +5104,8 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, Ex 43, 44, 45
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,22 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_477F4F93D44ABAEB52DAC3CEF1784B7EEFBDF254" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9CBF8C6-ED2F-4F70-A327-CE46CEF46189}"/>
   <bookViews>
-    <workbookView windowWidth="28245" windowHeight="12615"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="268">
   <si>
     <t>Order</t>
   </si>
@@ -825,15 +845,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -854,157 +870,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="9"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1029,194 +904,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1224,332 +913,59 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
+      <font>
+        <b/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1563,24 +979,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1590,43 +989,54 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" name="Order"/>
-    <tableColumn id="2" name="Planned Date"/>
-    <tableColumn id="3" name="Task Type"/>
-    <tableColumn id="4" name="Phase"/>
-    <tableColumn id="5" name="Section(s)"/>
-    <tableColumn id="6" name="Task"/>
-    <tableColumn id="7" name="Exercise"/>
-    <tableColumn id="8" name="Related Result / Reason"/>
-    <tableColumn id="9" name="Prerequisite"/>
-    <tableColumn id="10" name="Proceed Gate"/>
-    <tableColumn id="11" name="Actual Start"/>
-    <tableColumn id="12" name="Actual End"/>
-    <tableColumn id="13" name="First-pass Status"/>
-    <tableColumn id="14" name="Key Blocker"/>
-    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
-    <tableColumn id="16" name="Redo Result"/>
-    <tableColumn id="17" name="Proceed?"/>
-    <tableColumn id="18" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
+      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
+      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" name="First-pass Status"/>
-    <tableColumn id="2" name="Meaning"/>
-    <tableColumn id="3" name="Recommended Action"/>
-    <tableColumn id="4" name="Redo Offset Days"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1775,25 +1185,25 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="37.45" customWidth="1"/>
+    <col min="6" max="6" width="37.5" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="19.9083333333333" customWidth="1"/>
-    <col min="9" max="9" width="21.725" customWidth="1"/>
-    <col min="10" max="10" width="18.3666666666667" customWidth="1"/>
-    <col min="11" max="11" width="17.9083333333333" customWidth="1"/>
+    <col min="8" max="8" width="19.875" customWidth="1"/>
+    <col min="9" max="9" width="21.75" customWidth="1"/>
+    <col min="10" max="10" width="18.375" customWidth="1"/>
+    <col min="11" max="11" width="17.875" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
     <col min="14" max="14" width="28" customWidth="1"/>
@@ -1804,7 +1214,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.15" customHeight="1" spans="1:19">
+    <row r="1" spans="1:19" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1863,7 +1273,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="42.75" spans="1:19">
+    <row r="2" spans="1:19" ht="54">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1904,7 +1314,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" ht="42.75" spans="1:19">
+    <row r="3" spans="1:19" ht="54">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1945,7 +1355,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" ht="28.5" spans="1:19">
+    <row r="4" spans="1:19" ht="27">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1991,7 +1401,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" ht="28.5" spans="1:19">
+    <row r="5" spans="1:19" ht="27">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2042,7 +1452,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" ht="28.5" spans="1:19">
+    <row r="6" spans="1:19" ht="27">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2093,7 +1503,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" ht="28.5" spans="1:19">
+    <row r="7" spans="1:19" ht="27">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2144,7 +1554,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" ht="28.5" spans="1:19">
+    <row r="8" spans="1:19" ht="27">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2195,7 +1605,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" ht="28.5" spans="1:19">
+    <row r="9" spans="1:19" ht="27">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2246,7 +1656,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" ht="27">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2297,7 +1707,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" ht="28.5" spans="1:19">
+    <row r="11" spans="1:19" ht="27">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2348,7 +1758,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" ht="57" spans="1:19">
+    <row r="12" spans="1:19" ht="54">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2397,7 +1807,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" ht="42.75" spans="1:19">
+    <row r="13" spans="1:19" ht="40.5">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2439,7 +1849,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" ht="28.5" spans="1:19">
+    <row r="14" spans="1:19" ht="40.5">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2490,7 +1900,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" ht="28.5" spans="1:19">
+    <row r="15" spans="1:19" ht="27">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2541,7 +1951,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" ht="28.5" spans="1:19">
+    <row r="16" spans="1:19" ht="27">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2592,7 +2002,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" ht="28.5" spans="1:19">
+    <row r="17" spans="1:19" ht="40.5">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2643,7 +2053,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" ht="28.5" spans="1:19">
+    <row r="18" spans="1:19" ht="40.5">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2696,7 +2106,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" ht="28.5" spans="1:19">
+    <row r="19" spans="1:19" ht="27">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2747,7 +2157,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" ht="28.5" spans="1:19">
+    <row r="20" spans="1:19" ht="27">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2798,7 +2208,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" ht="57" spans="1:19">
+    <row r="21" spans="1:19" ht="67.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2844,7 +2254,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" ht="42.75" spans="1:19">
+    <row r="22" spans="1:19" ht="40.5">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2886,7 +2296,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" ht="42.75" spans="1:19">
+    <row r="23" spans="1:19" ht="40.5">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2928,7 +2338,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" ht="28.5" spans="1:19">
+    <row r="24" spans="1:19" ht="40.5">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2978,7 +2388,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" ht="28.5" spans="1:19">
+    <row r="25" spans="1:19" ht="27">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -3029,7 +2439,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" ht="28.5" spans="1:19">
+    <row r="26" spans="1:19" ht="27">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -3080,7 +2490,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" ht="28.5" spans="1:19">
+    <row r="27" spans="1:19" ht="40.5">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -3133,7 +2543,7 @@
       </c>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" ht="42.75" spans="1:19">
+    <row r="28" spans="1:19" ht="40.5">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -3179,7 +2589,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" ht="42.75" spans="1:19">
+    <row r="29" spans="1:19" ht="54">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3221,7 +2631,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" ht="28.5" spans="1:19">
+    <row r="30" spans="1:19" ht="40.5">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3263,7 +2673,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" ht="42.75" spans="1:19">
+    <row r="31" spans="1:19" ht="40.5">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3314,7 +2724,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" ht="42.75" spans="1:19">
+    <row r="32" spans="1:19" ht="40.5">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -3365,7 +2775,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" ht="42.75" spans="1:19">
+    <row r="33" spans="1:19" ht="40.5">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3416,7 +2826,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" ht="42.75" spans="1:19">
+    <row r="34" spans="1:19" ht="40.5">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -3467,7 +2877,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" ht="42.75" spans="1:19">
+    <row r="35" spans="1:19" ht="40.5">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3518,7 +2928,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" ht="42.75" spans="1:19">
+    <row r="36" spans="1:19" ht="40.5">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -3550,9 +2960,9 @@
       <c r="K36" s="7">
         <v>46226</v>
       </c>
-      <c r="L36" s="7" t="str">
+      <c r="L36" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46231</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>55</v>
@@ -3562,12 +2972,14 @@
         <f>IF(AND($C36="Exercise",$K36&lt;&gt;"",$M36&lt;&gt;""),$K36+VLOOKUP($M36,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46228</v>
       </c>
-      <c r="P36" s="7"/>
+      <c r="P36" s="7">
+        <v>46231</v>
+      </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" ht="42.75" spans="1:19">
+    <row r="37" spans="1:19" ht="40.5">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3618,7 +3030,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" ht="42.75" spans="1:19">
+    <row r="38" spans="1:19" ht="40.5">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3667,7 +3079,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" ht="42.75" spans="1:19">
+    <row r="39" spans="1:19" ht="40.5">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3696,23 +3108,27 @@
         <v>136</v>
       </c>
       <c r="J39" s="6"/>
-      <c r="K39" s="7"/>
+      <c r="K39" s="7">
+        <v>46231</v>
+      </c>
       <c r="L39" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M39" s="6"/>
+      <c r="M39" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="N39" s="6"/>
-      <c r="O39" s="7" t="str">
+      <c r="O39" s="7">
         <f>IF(AND($C39="Exercise",$K39&lt;&gt;"",$M39&lt;&gt;""),$K39+VLOOKUP($M39,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46233</v>
       </c>
       <c r="P39" s="7"/>
       <c r="Q39" s="6"/>
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" ht="42.75" spans="1:19">
+    <row r="40" spans="1:19" ht="40.5">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3741,23 +3157,27 @@
         <v>136</v>
       </c>
       <c r="J40" s="6"/>
-      <c r="K40" s="7"/>
+      <c r="K40" s="7">
+        <v>46234</v>
+      </c>
       <c r="L40" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M40" s="6"/>
+      <c r="M40" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N40" s="6"/>
-      <c r="O40" s="7" t="str">
+      <c r="O40" s="7">
         <f>IF(AND($C40="Exercise",$K40&lt;&gt;"",$M40&lt;&gt;""),$K40+VLOOKUP($M40,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46236</v>
       </c>
       <c r="P40" s="7"/>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" ht="42.75" spans="1:19">
+    <row r="41" spans="1:19" ht="54">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3802,7 +3222,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" ht="42.75" spans="1:19">
+    <row r="42" spans="1:19" ht="54">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3843,7 +3263,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" ht="42.75" spans="1:19">
+    <row r="43" spans="1:19" ht="40.5">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3884,7 +3304,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" ht="42.75" spans="1:19">
+    <row r="44" spans="1:19" ht="40.5">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3929,7 +3349,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" ht="42.75" spans="1:19">
+    <row r="45" spans="1:19" ht="40.5">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3974,7 +3394,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" ht="42.75" spans="1:19">
+    <row r="46" spans="1:19" ht="40.5">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -4019,7 +3439,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" ht="42.75" spans="1:19">
+    <row r="47" spans="1:19" ht="40.5">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -4064,7 +3484,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" ht="42.75" spans="1:19">
+    <row r="48" spans="1:19" ht="40.5">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -4109,7 +3529,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" ht="42.75" spans="1:19">
+    <row r="49" spans="1:19" ht="40.5">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -4154,7 +3574,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" ht="42.75" spans="1:19">
+    <row r="50" spans="1:19" ht="40.5">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -4199,7 +3619,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" ht="42.75" spans="1:19">
+    <row r="51" spans="1:19" ht="40.5">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -4244,7 +3664,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" ht="42.75" spans="1:19">
+    <row r="52" spans="1:19" ht="40.5">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -4289,7 +3709,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" ht="42.75" spans="1:19">
+    <row r="53" spans="1:19" ht="40.5">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -4334,7 +3754,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" ht="42.75" spans="1:19">
+    <row r="54" spans="1:19" ht="40.5">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -4379,7 +3799,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" ht="42.75" spans="1:19">
+    <row r="55" spans="1:19" ht="40.5">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -4424,7 +3844,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" ht="42.75" spans="1:19">
+    <row r="56" spans="1:19" ht="54">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -4469,7 +3889,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" ht="57" spans="1:19">
+    <row r="57" spans="1:19" ht="67.5">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -4510,7 +3930,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" ht="28.5" spans="1:19">
+    <row r="58" spans="1:19" ht="40.5">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4555,7 +3975,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" ht="28.5" spans="1:19">
+    <row r="59" spans="1:19" ht="27">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4600,7 +4020,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" ht="28.5" spans="1:19">
+    <row r="60" spans="1:19" ht="27">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4645,7 +4065,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" ht="28.5" spans="1:19">
+    <row r="61" spans="1:19" ht="27">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4690,7 +4110,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" ht="28.5" spans="1:19">
+    <row r="62" spans="1:19" ht="27">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4735,7 +4155,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" ht="42.75" spans="1:19">
+    <row r="63" spans="1:19" ht="54">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4776,7 +4196,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" ht="57" spans="1:19">
+    <row r="64" spans="1:19" ht="54">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4818,35 +4238,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64">
+    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64">
+    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
+  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4854,22 +4274,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" spans="1:2">
+    <row r="1" spans="1:2" ht="27">
       <c r="A1" s="1" t="s">
         <v>239</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" ht="28.5" spans="1:2">
+    <row r="2" spans="1:2" ht="27">
       <c r="A2" s="3" t="s">
         <v>240</v>
       </c>
@@ -4881,7 +4300,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" ht="15" spans="1:2">
+    <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>242</v>
       </c>
@@ -4890,7 +4309,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="15" spans="1:2">
+    <row r="5" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>243</v>
       </c>
@@ -4899,7 +4318,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="15" spans="1:2">
+    <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>244</v>
       </c>
@@ -4908,7 +4327,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" ht="15" spans="1:2">
+    <row r="7" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>245</v>
       </c>
@@ -4917,7 +4336,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="15" spans="1:2">
+    <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>246</v>
       </c>
@@ -4926,29 +4345,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15" spans="1:2">
+    <row r="9" spans="1:2" ht="27">
       <c r="A9" s="5" t="s">
         <v>247</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" ht="15" spans="1:2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="27">
       <c r="A10" s="5" t="s">
         <v>248</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" ht="15" spans="1:2">
+    <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>249</v>
       </c>
@@ -4957,16 +4376,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="15" spans="1:2">
+    <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Spark")</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" ht="15" spans="1:2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -4975,20 +4394,20 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" ht="15" spans="1:2">
+    <row r="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" ht="15" spans="1:2">
+    <row r="17" spans="1:2" ht="27">
       <c r="A17" s="5" t="s">
         <v>250</v>
       </c>
@@ -4996,7 +4415,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="18" ht="15" spans="1:2">
+    <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>252</v>
       </c>
@@ -5005,16 +4424,15 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -5022,7 +4440,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:4">
+    <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -5092,7 +4510,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>265</v>
       </c>
@@ -5104,8 +4522,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, a bunch of exercises
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_477F4F93D44ABAEB52DAC3CEF1784B7EEFBDF254" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9CBF8C6-ED2F-4F70-A327-CE46CEF46189}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_477F4F93D44ABAEB52DAC3CEF1784B7EEFBDF254" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4F6B5E8-6F91-4006-B08F-436849A47C93}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="268">
   <si>
     <t>Order</t>
   </si>
@@ -3111,9 +3111,9 @@
       <c r="K39" s="7">
         <v>46231</v>
       </c>
-      <c r="L39" s="7" t="str">
+      <c r="L39" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46235</v>
       </c>
       <c r="M39" s="6" t="s">
         <v>55</v>
@@ -3123,7 +3123,9 @@
         <f>IF(AND($C39="Exercise",$K39&lt;&gt;"",$M39&lt;&gt;""),$K39+VLOOKUP($M39,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46233</v>
       </c>
-      <c r="P39" s="7"/>
+      <c r="P39" s="7">
+        <v>46235</v>
+      </c>
       <c r="Q39" s="6"/>
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
@@ -3206,7 +3208,9 @@
       <c r="J41" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="K41" s="7"/>
+      <c r="K41" s="7">
+        <v>46235</v>
+      </c>
       <c r="L41" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3333,16 +3337,20 @@
         <v>177</v>
       </c>
       <c r="J44" s="6"/>
-      <c r="K44" s="7"/>
+      <c r="K44" s="7">
+        <v>46242</v>
+      </c>
       <c r="L44" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M44" s="6"/>
+      <c r="M44" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N44" s="6"/>
-      <c r="O44" s="7" t="str">
+      <c r="O44" s="7">
         <f>IF(AND($C44="Exercise",$K44&lt;&gt;"",$M44&lt;&gt;""),$K44+VLOOKUP($M44,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46244</v>
       </c>
       <c r="P44" s="7"/>
       <c r="Q44" s="6"/>
@@ -3378,16 +3386,20 @@
         <v>177</v>
       </c>
       <c r="J45" s="6"/>
-      <c r="K45" s="7"/>
+      <c r="K45" s="7">
+        <v>46243</v>
+      </c>
       <c r="L45" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M45" s="6"/>
+      <c r="M45" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N45" s="6"/>
-      <c r="O45" s="7" t="str">
+      <c r="O45" s="7">
         <f>IF(AND($C45="Exercise",$K45&lt;&gt;"",$M45&lt;&gt;""),$K45+VLOOKUP($M45,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46245</v>
       </c>
       <c r="P45" s="7"/>
       <c r="Q45" s="6"/>
@@ -4351,7 +4363,7 @@
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="27">
@@ -4360,7 +4372,7 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4391,7 +4403,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:2">

</xml_diff>

<commit_message>
Chap 7, Ex 19
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="268">
   <si>
     <t>Order</t>
   </si>
@@ -827,10 +827,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="23">
@@ -861,7 +861,30 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -876,6 +899,28 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -906,39 +951,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -952,39 +965,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="13"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -999,6 +984,21 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1031,7 +1031,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1043,13 +1043,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1061,13 +1055,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1085,19 +1073,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1109,13 +1127,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1133,49 +1175,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1187,31 +1199,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1228,8 +1228,32 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1253,7 +1277,22 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4"/>
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1283,190 +1322,151 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="27" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -4134,9 +4134,9 @@
       <c r="K48" s="7">
         <v>46246</v>
       </c>
-      <c r="L48" s="7" t="str">
+      <c r="L48" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46248</v>
       </c>
       <c r="M48" s="6" t="s">
         <v>39</v>
@@ -4146,7 +4146,9 @@
         <f>IF(AND($C48="Exercise",$K48&lt;&gt;"",$M48&lt;&gt;""),$K48+VLOOKUP($M48,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46248</v>
       </c>
-      <c r="P48" s="7"/>
+      <c r="P48" s="7">
+        <v>46248</v>
+      </c>
       <c r="Q48" s="6"/>
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
@@ -4229,16 +4231,20 @@
         <v>177</v>
       </c>
       <c r="J50" s="6"/>
-      <c r="K50" s="7"/>
+      <c r="K50" s="7">
+        <v>46248</v>
+      </c>
       <c r="L50" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M50" s="6"/>
+      <c r="M50" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N50" s="6"/>
-      <c r="O50" s="7" t="str">
+      <c r="O50" s="7">
         <f>IF(AND($C50="Exercise",$K50&lt;&gt;"",$M50&lt;&gt;""),$K50+VLOOKUP($M50,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46250</v>
       </c>
       <c r="P50" s="7"/>
       <c r="Q50" s="6"/>
@@ -4978,7 +4984,7 @@
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" ht="15" spans="1:2">
@@ -4987,7 +4993,7 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -5018,7 +5024,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" ht="15" spans="1:2">

</xml_diff>

<commit_message>
Chap 7, Ex 20, 26
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,22 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8372600-3BD6-4E8F-8A6C-09DD99FE512F}"/>
   <bookViews>
-    <workbookView windowWidth="19935" windowHeight="7935"/>
+    <workbookView xWindow="29790" yWindow="2820" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="268">
   <si>
     <t>Order</t>
   </si>
@@ -825,15 +845,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -854,157 +870,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
+      <sz val="9"/>
+      <name val="Carlito"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1029,194 +904,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1224,332 +913,59 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
+      <font>
+        <b/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1563,24 +979,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1590,43 +989,54 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" name="Order"/>
-    <tableColumn id="2" name="Planned Date"/>
-    <tableColumn id="3" name="Task Type"/>
-    <tableColumn id="4" name="Phase"/>
-    <tableColumn id="5" name="Section(s)"/>
-    <tableColumn id="6" name="Task"/>
-    <tableColumn id="7" name="Exercise"/>
-    <tableColumn id="8" name="Related Result / Reason"/>
-    <tableColumn id="9" name="Prerequisite"/>
-    <tableColumn id="10" name="Proceed Gate"/>
-    <tableColumn id="11" name="Actual Start"/>
-    <tableColumn id="12" name="Actual End"/>
-    <tableColumn id="13" name="First-pass Status"/>
-    <tableColumn id="14" name="Key Blocker"/>
-    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
-    <tableColumn id="16" name="Redo Result"/>
-    <tableColumn id="17" name="Proceed?"/>
-    <tableColumn id="18" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
+      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
+      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" name="First-pass Status"/>
-    <tableColumn id="2" name="Meaning"/>
-    <tableColumn id="3" name="Recommended Action"/>
-    <tableColumn id="4" name="Redo Offset Days"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1775,14 +1185,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1804,7 +1214,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.1" customHeight="1" spans="1:19">
+    <row r="1" spans="1:19" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1863,7 +1273,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="42.75" spans="1:19">
+    <row r="2" spans="1:19" ht="54">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1904,7 +1314,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" ht="42.75" spans="1:19">
+    <row r="3" spans="1:19" ht="54">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1945,7 +1355,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" ht="28.5" spans="1:19">
+    <row r="4" spans="1:19" ht="27">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1991,7 +1401,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" ht="28.5" spans="1:19">
+    <row r="5" spans="1:19" ht="27">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2042,7 +1452,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" ht="28.5" spans="1:19">
+    <row r="6" spans="1:19" ht="27">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2093,7 +1503,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" ht="28.5" spans="1:19">
+    <row r="7" spans="1:19" ht="27">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2144,7 +1554,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" ht="28.5" spans="1:19">
+    <row r="8" spans="1:19" ht="27">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2195,7 +1605,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" ht="28.5" spans="1:19">
+    <row r="9" spans="1:19" ht="27">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2246,7 +1656,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" ht="27">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2297,7 +1707,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" ht="28.5" spans="1:19">
+    <row r="11" spans="1:19" ht="27">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2348,7 +1758,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" ht="57" spans="1:19">
+    <row r="12" spans="1:19" ht="54">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2397,7 +1807,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" ht="42.75" spans="1:19">
+    <row r="13" spans="1:19" ht="40.5">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2439,7 +1849,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" ht="28.5" spans="1:19">
+    <row r="14" spans="1:19" ht="40.5">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2490,7 +1900,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" ht="28.5" spans="1:19">
+    <row r="15" spans="1:19" ht="27">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2541,7 +1951,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" ht="28.5" spans="1:19">
+    <row r="16" spans="1:19" ht="27">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2592,7 +2002,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" ht="28.5" spans="1:19">
+    <row r="17" spans="1:19" ht="40.5">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2643,7 +2053,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" ht="28.5" spans="1:19">
+    <row r="18" spans="1:19" ht="40.5">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2696,7 +2106,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" ht="28.5" spans="1:19">
+    <row r="19" spans="1:19" ht="27">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2747,7 +2157,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" ht="28.5" spans="1:19">
+    <row r="20" spans="1:19" ht="27">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2798,7 +2208,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" ht="57" spans="1:19">
+    <row r="21" spans="1:19" ht="67.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2844,7 +2254,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" ht="42.75" spans="1:19">
+    <row r="22" spans="1:19" ht="40.5">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2886,7 +2296,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" ht="42.75" spans="1:19">
+    <row r="23" spans="1:19" ht="40.5">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2928,7 +2338,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" ht="28.5" spans="1:19">
+    <row r="24" spans="1:19" ht="40.5">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2978,7 +2388,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" ht="28.5" spans="1:19">
+    <row r="25" spans="1:19" ht="27">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -3029,7 +2439,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" ht="28.5" spans="1:19">
+    <row r="26" spans="1:19" ht="27">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -3080,7 +2490,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" ht="28.5" spans="1:19">
+    <row r="27" spans="1:19" ht="40.5">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -3133,7 +2543,7 @@
       </c>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" ht="42.75" spans="1:19">
+    <row r="28" spans="1:19" ht="40.5">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -3179,7 +2589,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" ht="42.75" spans="1:19">
+    <row r="29" spans="1:19" ht="54">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3221,7 +2631,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" ht="28.5" spans="1:19">
+    <row r="30" spans="1:19" ht="40.5">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -3263,7 +2673,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" ht="28.5" spans="1:19">
+    <row r="31" spans="1:19" ht="40.5">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3314,7 +2724,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" ht="28.5" spans="1:19">
+    <row r="32" spans="1:19" ht="40.5">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -3365,7 +2775,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" ht="28.5" spans="1:19">
+    <row r="33" spans="1:19" ht="40.5">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3416,7 +2826,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" ht="28.5" spans="1:19">
+    <row r="34" spans="1:19" ht="40.5">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -3467,7 +2877,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" ht="28.5" spans="1:19">
+    <row r="35" spans="1:19" ht="40.5">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3518,7 +2928,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" ht="28.5" spans="1:19">
+    <row r="36" spans="1:19" ht="40.5">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -3569,7 +2979,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" ht="28.5" spans="1:19">
+    <row r="37" spans="1:19" ht="40.5">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3620,7 +3030,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" ht="28.5" spans="1:19">
+    <row r="38" spans="1:19" ht="40.5">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3669,7 +3079,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" ht="28.5" spans="1:19">
+    <row r="39" spans="1:19" ht="40.5">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3720,7 +3130,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" ht="28.5" spans="1:19">
+    <row r="40" spans="1:19" ht="40.5">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3769,7 +3179,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" ht="42.75" spans="1:19">
+    <row r="41" spans="1:19" ht="54">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3816,7 +3226,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" ht="42.75" spans="1:19">
+    <row r="42" spans="1:19" ht="54">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3857,7 +3267,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" ht="42.75" spans="1:19">
+    <row r="43" spans="1:19" ht="40.5">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3898,7 +3308,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" ht="28.5" spans="1:19">
+    <row r="44" spans="1:19" ht="40.5">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3949,7 +3359,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" ht="28.5" spans="1:19">
+    <row r="45" spans="1:19" ht="40.5">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -4000,7 +3410,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" ht="28.5" spans="1:19">
+    <row r="46" spans="1:19" ht="40.5">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -4051,7 +3461,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" ht="28.5" spans="1:19">
+    <row r="47" spans="1:19" ht="40.5">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -4102,7 +3512,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" ht="28.5" spans="1:19">
+    <row r="48" spans="1:19" ht="40.5">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -4153,7 +3563,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" ht="28.5" spans="1:19">
+    <row r="49" spans="1:19" ht="40.5">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -4185,9 +3595,9 @@
       <c r="K49" s="7">
         <v>46247</v>
       </c>
-      <c r="L49" s="7" t="str">
+      <c r="L49" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46249</v>
       </c>
       <c r="M49" s="6" t="s">
         <v>30</v>
@@ -4197,12 +3607,14 @@
         <f>IF(AND($C49="Exercise",$K49&lt;&gt;"",$M49&lt;&gt;""),$K49+VLOOKUP($M49,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46249</v>
       </c>
-      <c r="P49" s="7"/>
+      <c r="P49" s="7">
+        <v>46249</v>
+      </c>
       <c r="Q49" s="6"/>
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" ht="28.5" spans="1:19">
+    <row r="50" spans="1:19" ht="40.5">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -4251,7 +3663,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" ht="28.5" spans="1:19">
+    <row r="51" spans="1:19" ht="40.5">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -4280,23 +3692,27 @@
         <v>177</v>
       </c>
       <c r="J51" s="6"/>
-      <c r="K51" s="7"/>
+      <c r="K51" s="7">
+        <v>46248</v>
+      </c>
       <c r="L51" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M51" s="6"/>
+      <c r="M51" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N51" s="6"/>
-      <c r="O51" s="7" t="str">
+      <c r="O51" s="7">
         <f>IF(AND($C51="Exercise",$K51&lt;&gt;"",$M51&lt;&gt;""),$K51+VLOOKUP($M51,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46250</v>
       </c>
       <c r="P51" s="7"/>
       <c r="Q51" s="6"/>
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" ht="28.5" spans="1:19">
+    <row r="52" spans="1:19" ht="40.5">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -4325,23 +3741,27 @@
         <v>177</v>
       </c>
       <c r="J52" s="6"/>
-      <c r="K52" s="7"/>
+      <c r="K52" s="7">
+        <v>46249</v>
+      </c>
       <c r="L52" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M52" s="6"/>
+      <c r="M52" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N52" s="6"/>
-      <c r="O52" s="7" t="str">
+      <c r="O52" s="7">
         <f>IF(AND($C52="Exercise",$K52&lt;&gt;"",$M52&lt;&gt;""),$K52+VLOOKUP($M52,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46251</v>
       </c>
       <c r="P52" s="7"/>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" ht="28.5" spans="1:19">
+    <row r="53" spans="1:19" ht="40.5">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -4386,7 +3806,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" ht="28.5" spans="1:19">
+    <row r="54" spans="1:19" ht="40.5">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -4431,7 +3851,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" ht="28.5" spans="1:19">
+    <row r="55" spans="1:19" ht="40.5">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -4476,7 +3896,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" ht="42.75" spans="1:19">
+    <row r="56" spans="1:19" ht="54">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -4521,7 +3941,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" ht="57" spans="1:19">
+    <row r="57" spans="1:19" ht="67.5">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -4562,7 +3982,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" ht="28.5" spans="1:19">
+    <row r="58" spans="1:19" ht="40.5">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4607,7 +4027,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" ht="28.5" spans="1:19">
+    <row r="59" spans="1:19" ht="27">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4652,7 +4072,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" ht="28.5" spans="1:19">
+    <row r="60" spans="1:19" ht="27">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4697,7 +4117,7 @@
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" ht="28.5" spans="1:19">
+    <row r="61" spans="1:19" ht="27">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4742,7 +4162,7 @@
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" ht="28.5" spans="1:19">
+    <row r="62" spans="1:19" ht="27">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4787,7 +4207,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" ht="42.75" spans="1:19">
+    <row r="63" spans="1:19" ht="54">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4828,7 +4248,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" ht="57" spans="1:19">
+    <row r="64" spans="1:19" ht="54">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4870,35 +4290,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64">
+    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64">
+    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
+  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4906,22 +4326,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" spans="1:2">
+    <row r="1" spans="1:2" ht="27">
       <c r="A1" s="1" t="s">
         <v>239</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" ht="28.5" spans="1:2">
+    <row r="2" spans="1:2" ht="27">
       <c r="A2" s="3" t="s">
         <v>240</v>
       </c>
@@ -4933,7 +4352,7 @@
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" ht="15" spans="1:2">
+    <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
         <v>242</v>
       </c>
@@ -4942,7 +4361,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="15" spans="1:2">
+    <row r="5" spans="1:2">
       <c r="A5" s="5" t="s">
         <v>243</v>
       </c>
@@ -4951,7 +4370,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="15" spans="1:2">
+    <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
         <v>244</v>
       </c>
@@ -4960,7 +4379,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" ht="15" spans="1:2">
+    <row r="7" spans="1:2">
       <c r="A7" s="5" t="s">
         <v>245</v>
       </c>
@@ -4969,7 +4388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="15" spans="1:2">
+    <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
         <v>246</v>
       </c>
@@ -4978,29 +4397,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15" spans="1:2">
+    <row r="9" spans="1:2" ht="27">
       <c r="A9" s="5" t="s">
         <v>247</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" ht="15" spans="1:2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="27">
       <c r="A10" s="5" t="s">
         <v>248</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" ht="15" spans="1:2">
+    <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
         <v>249</v>
       </c>
@@ -5009,7 +4428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="15" spans="1:2">
+    <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -5018,7 +4437,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" ht="15" spans="1:2">
+    <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -5027,20 +4446,20 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" ht="15" spans="1:2">
+    <row r="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" ht="15" spans="1:2">
+    <row r="17" spans="1:2" ht="27">
       <c r="A17" s="5" t="s">
         <v>250</v>
       </c>
@@ -5048,7 +4467,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="18" ht="15" spans="1:2">
+    <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
         <v>252</v>
       </c>
@@ -5057,16 +4476,15 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -5074,7 +4492,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:4">
+    <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -5144,7 +4562,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>265</v>
       </c>
@@ -5156,8 +4574,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Chap 7, Ex 33. 36
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8372600-3BD6-4E8F-8A6C-09DD99FE512F}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BCDB5FC-2D57-41B4-8868-4EBF477326FF}"/>
   <bookViews>
-    <workbookView xWindow="29790" yWindow="2820" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1935" yWindow="2865" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="269">
   <si>
     <t>Order</t>
   </si>
@@ -840,6 +840,10 @@
   </si>
   <si>
     <t>Suggested Redo Date = Actual Start + offset. Actual End is automatically filled from Actual Redo Date.</t>
+  </si>
+  <si>
+    <t>Same as Ex 13</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -847,7 +851,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -936,7 +940,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3790,16 +3794,20 @@
         <v>177</v>
       </c>
       <c r="J53" s="6"/>
-      <c r="K53" s="7"/>
+      <c r="K53" s="7">
+        <v>46249</v>
+      </c>
       <c r="L53" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M53" s="6"/>
+      <c r="M53" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N53" s="6"/>
-      <c r="O53" s="7" t="str">
+      <c r="O53" s="7">
         <f>IF(AND($C53="Exercise",$K53&lt;&gt;"",$M53&lt;&gt;""),$K53+VLOOKUP($M53,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46251</v>
       </c>
       <c r="P53" s="7"/>
       <c r="Q53" s="6"/>
@@ -3835,16 +3843,20 @@
         <v>177</v>
       </c>
       <c r="J54" s="6"/>
-      <c r="K54" s="7"/>
+      <c r="K54" s="7">
+        <v>46249</v>
+      </c>
       <c r="L54" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M54" s="6"/>
+      <c r="M54" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N54" s="6"/>
-      <c r="O54" s="7" t="str">
+      <c r="O54" s="7">
         <f>IF(AND($C54="Exercise",$K54&lt;&gt;"",$M54&lt;&gt;""),$K54+VLOOKUP($M54,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46251</v>
       </c>
       <c r="P54" s="7"/>
       <c r="Q54" s="6"/>
@@ -3880,7 +3892,9 @@
         <v>177</v>
       </c>
       <c r="J55" s="6"/>
-      <c r="K55" s="7"/>
+      <c r="K55" s="7" t="s">
+        <v>268</v>
+      </c>
       <c r="L55" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4452,7 +4466,7 @@
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:2">

</xml_diff>

<commit_message>
Chap 7 Ex 24
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCDD8A4F-870E-443E-8B20-EB70A9AD24DD}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E50DD782-8A86-432C-8A62-4815BCF539B2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="269">
   <si>
     <t>Order</t>
   </si>
@@ -3650,9 +3650,9 @@
       <c r="K50" s="7">
         <v>46248</v>
       </c>
-      <c r="L50" s="7" t="str">
+      <c r="L50" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46250</v>
       </c>
       <c r="M50" s="6" t="s">
         <v>39</v>
@@ -3662,7 +3662,9 @@
         <f>IF(AND($C50="Exercise",$K50&lt;&gt;"",$M50&lt;&gt;""),$K50+VLOOKUP($M50,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46250</v>
       </c>
-      <c r="P50" s="7"/>
+      <c r="P50" s="7">
+        <v>46250</v>
+      </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
@@ -3699,9 +3701,9 @@
       <c r="K51" s="7">
         <v>46248</v>
       </c>
-      <c r="L51" s="7" t="str">
+      <c r="L51" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46250</v>
       </c>
       <c r="M51" s="6" t="s">
         <v>30</v>
@@ -3711,7 +3713,9 @@
         <f>IF(AND($C51="Exercise",$K51&lt;&gt;"",$M51&lt;&gt;""),$K51+VLOOKUP($M51,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46250</v>
       </c>
-      <c r="P51" s="7"/>
+      <c r="P51" s="7">
+        <v>46250</v>
+      </c>
       <c r="Q51" s="6"/>
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
@@ -3748,9 +3752,9 @@
       <c r="K52" s="7">
         <v>46249</v>
       </c>
-      <c r="L52" s="7" t="str">
+      <c r="L52" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46253</v>
       </c>
       <c r="M52" s="6" t="s">
         <v>30</v>
@@ -3760,7 +3764,9 @@
         <f>IF(AND($C52="Exercise",$K52&lt;&gt;"",$M52&lt;&gt;""),$K52+VLOOKUP($M52,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46251</v>
       </c>
-      <c r="P52" s="7"/>
+      <c r="P52" s="7">
+        <v>46253</v>
+      </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
@@ -3797,9 +3803,9 @@
       <c r="K53" s="7">
         <v>46249</v>
       </c>
-      <c r="L53" s="7" t="str">
+      <c r="L53" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46253</v>
       </c>
       <c r="M53" s="6" t="s">
         <v>30</v>
@@ -3809,7 +3815,9 @@
         <f>IF(AND($C53="Exercise",$K53&lt;&gt;"",$M53&lt;&gt;""),$K53+VLOOKUP($M53,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46251</v>
       </c>
-      <c r="P53" s="7"/>
+      <c r="P53" s="7">
+        <v>46253</v>
+      </c>
       <c r="Q53" s="6"/>
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
@@ -3846,9 +3854,9 @@
       <c r="K54" s="7">
         <v>46249</v>
       </c>
-      <c r="L54" s="7" t="str">
+      <c r="L54" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46253</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>30</v>
@@ -3858,7 +3866,9 @@
         <f>IF(AND($C54="Exercise",$K54&lt;&gt;"",$M54&lt;&gt;""),$K54+VLOOKUP($M54,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46251</v>
       </c>
-      <c r="P54" s="7"/>
+      <c r="P54" s="7">
+        <v>46253</v>
+      </c>
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
@@ -4029,18 +4039,24 @@
         <v>219</v>
       </c>
       <c r="J58" s="6"/>
-      <c r="K58" s="7"/>
-      <c r="L58" s="7" t="str">
+      <c r="K58" s="7">
+        <v>46251</v>
+      </c>
+      <c r="L58" s="7">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="M58" s="6"/>
+        <v>46264</v>
+      </c>
+      <c r="M58" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="N58" s="6"/>
-      <c r="O58" s="7" t="str">
+      <c r="O58" s="7">
         <f>IF(AND($C58="Exercise",$K58&lt;&gt;"",$M58&lt;&gt;""),$K58+VLOOKUP($M58,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="P58" s="7"/>
+        <v>46253</v>
+      </c>
+      <c r="P58" s="7">
+        <v>46264</v>
+      </c>
       <c r="Q58" s="6"/>
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
@@ -4421,7 +4437,7 @@
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="27">
@@ -4430,7 +4446,7 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4461,7 +4477,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Skeleton")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:2">

</xml_diff>

<commit_message>
Chap 7 Ex 25
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E50DD782-8A86-432C-8A62-4815BCF539B2}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{011A32EF-0172-45EB-B617-25EBEFE1C1DF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="269">
   <si>
     <t>Order</t>
   </si>
@@ -4090,16 +4090,20 @@
         <v>219</v>
       </c>
       <c r="J59" s="6"/>
-      <c r="K59" s="7"/>
+      <c r="K59" s="7">
+        <v>46265</v>
+      </c>
       <c r="L59" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M59" s="6"/>
+      <c r="M59" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N59" s="6"/>
-      <c r="O59" s="7" t="str">
+      <c r="O59" s="7">
         <f>IF(AND($C59="Exercise",$K59&lt;&gt;"",$M59&lt;&gt;""),$K59+VLOOKUP($M59,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46267</v>
       </c>
       <c r="P59" s="7"/>
       <c r="Q59" s="6"/>
@@ -4486,7 +4490,7 @@
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2">

</xml_diff>